<commit_message>
Conclui rotulagem B da amostra-ouro S02
</commit_message>
<xml_diff>
--- a/Lab03/data/amostra_ouro_s02/rotulos/rotulos_B.xlsx
+++ b/Lab03/data/amostra_ouro_s02/rotulos/rotulos_B.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instrucoes" sheetId="1" r:id="Rbd8681d431fa4ed9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="repositorios" sheetId="2" r:id="R7cadebd82741460d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="releases" sheetId="3" r:id="Rf539ce73e4584bbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instrucoes" sheetId="1" r:id="R311712dd755042c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="repositorios" sheetId="2" r:id="Raa0c890ff34849b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="releases" sheetId="3" r:id="Rc6af5f823276417f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48,13 +48,7 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -385,8 +379,12 @@
       <x:c r="B2" s="4" t="str">
         <x:v>https://github.com/Azure/AKS</x:v>
       </x:c>
-      <x:c r="C2" s="4"/>
-      <x:c r="D2" s="4"/>
+      <x:c r="C2" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="46" customHeight="1">
       <x:c r="A3" s="4" t="str">
@@ -395,8 +393,12 @@
       <x:c r="B3" s="4" t="str">
         <x:v>https://github.com/Chorus-AIDLC/Chorus</x:v>
       </x:c>
-      <x:c r="C3" s="4"/>
-      <x:c r="D3" s="4"/>
+      <x:c r="C3" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D3" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="46" customHeight="1">
       <x:c r="A4" s="4" t="str">
@@ -405,8 +407,12 @@
       <x:c r="B4" s="4" t="str">
         <x:v>https://github.com/Darkatse/TauriTavern</x:v>
       </x:c>
-      <x:c r="C4" s="4"/>
-      <x:c r="D4" s="4"/>
+      <x:c r="C4" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="46" customHeight="1">
       <x:c r="A5" s="4" t="str">
@@ -415,8 +421,12 @@
       <x:c r="B5" s="4" t="str">
         <x:v>https://github.com/GetStream/stream-chat-flutter</x:v>
       </x:c>
-      <x:c r="C5" s="4"/>
-      <x:c r="D5" s="4"/>
+      <x:c r="C5" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="4" t="str">
@@ -425,8 +435,12 @@
       <x:c r="B6" s="4" t="str">
         <x:v>https://github.com/MGdaasLab/WHartTest</x:v>
       </x:c>
-      <x:c r="C6" s="4"/>
-      <x:c r="D6" s="4"/>
+      <x:c r="C6" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="4" t="str">
@@ -435,8 +449,12 @@
       <x:c r="B7" s="4" t="str">
         <x:v>https://github.com/MaikuB/flutter_local_notifications</x:v>
       </x:c>
-      <x:c r="C7" s="4"/>
-      <x:c r="D7" s="4"/>
+      <x:c r="C7" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="4" t="str">
@@ -445,8 +463,12 @@
       <x:c r="B8" s="4" t="str">
         <x:v>https://github.com/NVIDIA-NeMo/Guardrails</x:v>
       </x:c>
-      <x:c r="C8" s="4"/>
-      <x:c r="D8" s="4"/>
+      <x:c r="C8" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="4" t="str">
@@ -455,8 +477,12 @@
       <x:c r="B9" s="4" t="str">
         <x:v>https://github.com/StuffAnThings/qbit_manage</x:v>
       </x:c>
-      <x:c r="C9" s="4"/>
-      <x:c r="D9" s="4"/>
+      <x:c r="C9" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="4" t="str">
@@ -465,8 +491,12 @@
       <x:c r="B10" s="4" t="str">
         <x:v>https://github.com/Sync-in/server</x:v>
       </x:c>
-      <x:c r="C10" s="4"/>
-      <x:c r="D10" s="4"/>
+      <x:c r="C10" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="4" t="str">
@@ -475,8 +505,12 @@
       <x:c r="B11" s="4" t="str">
         <x:v>https://github.com/TNG/ArchUnitNET</x:v>
       </x:c>
-      <x:c r="C11" s="4"/>
-      <x:c r="D11" s="4"/>
+      <x:c r="C11" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="4" t="str">
@@ -485,8 +519,12 @@
       <x:c r="B12" s="4" t="str">
         <x:v>https://github.com/Ylianst/MeshCentral</x:v>
       </x:c>
-      <x:c r="C12" s="4"/>
-      <x:c r="D12" s="4"/>
+      <x:c r="C12" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="4" t="str">
@@ -495,8 +533,12 @@
       <x:c r="B13" s="4" t="str">
         <x:v>https://github.com/actions/cache</x:v>
       </x:c>
-      <x:c r="C13" s="4"/>
-      <x:c r="D13" s="4"/>
+      <x:c r="C13" s="4" t="str">
+        <x:v>outro</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="4" t="str">
@@ -505,8 +547,12 @@
       <x:c r="B14" s="4" t="str">
         <x:v>https://github.com/agavra/tuicr</x:v>
       </x:c>
-      <x:c r="C14" s="4"/>
-      <x:c r="D14" s="4"/>
+      <x:c r="C14" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="4" t="str">
@@ -515,8 +561,12 @@
       <x:c r="B15" s="4" t="str">
         <x:v>https://github.com/apache/servicecomb-java-chassis</x:v>
       </x:c>
-      <x:c r="C15" s="4"/>
-      <x:c r="D15" s="4"/>
+      <x:c r="C15" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="4" t="str">
@@ -525,8 +575,12 @@
       <x:c r="B16" s="4" t="str">
         <x:v>https://github.com/apify/fingerprint-suite</x:v>
       </x:c>
-      <x:c r="C16" s="4"/>
-      <x:c r="D16" s="4"/>
+      <x:c r="C16" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="4" t="str">
@@ -535,8 +589,12 @@
       <x:c r="B17" s="4" t="str">
         <x:v>https://github.com/ardatan/graphql-tools</x:v>
       </x:c>
-      <x:c r="C17" s="4"/>
-      <x:c r="D17" s="4"/>
+      <x:c r="C17" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="4" t="str">
@@ -545,8 +603,12 @@
       <x:c r="B18" s="4" t="str">
         <x:v>https://github.com/ariebovenberg/whenever</x:v>
       </x:c>
-      <x:c r="C18" s="4"/>
-      <x:c r="D18" s="4"/>
+      <x:c r="C18" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="A19" s="4" t="str">
@@ -555,8 +617,12 @@
       <x:c r="B19" s="4" t="str">
         <x:v>https://github.com/arkime/arkime</x:v>
       </x:c>
-      <x:c r="C19" s="4"/>
-      <x:c r="D19" s="4"/>
+      <x:c r="C19" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="46" customHeight="1">
       <x:c r="A20" s="4" t="str">
@@ -565,8 +631,12 @@
       <x:c r="B20" s="4" t="str">
         <x:v>https://github.com/borgbase/vorta</x:v>
       </x:c>
-      <x:c r="C20" s="4"/>
-      <x:c r="D20" s="4"/>
+      <x:c r="C20" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="46" customHeight="1">
       <x:c r="A21" s="4" t="str">
@@ -575,8 +645,12 @@
       <x:c r="B21" s="4" t="str">
         <x:v>https://github.com/bpg/terraform-provider-proxmox</x:v>
       </x:c>
-      <x:c r="C21" s="4"/>
-      <x:c r="D21" s="4"/>
+      <x:c r="C21" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="46" customHeight="1">
       <x:c r="A22" s="4" t="str">
@@ -585,8 +659,12 @@
       <x:c r="B22" s="4" t="str">
         <x:v>https://github.com/bubbuild/bub</x:v>
       </x:c>
-      <x:c r="C22" s="4"/>
-      <x:c r="D22" s="4"/>
+      <x:c r="C22" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="46" customHeight="1">
       <x:c r="A23" s="4" t="str">
@@ -595,8 +673,12 @@
       <x:c r="B23" s="4" t="str">
         <x:v>https://github.com/caezium/burrow</x:v>
       </x:c>
-      <x:c r="C23" s="4"/>
-      <x:c r="D23" s="4"/>
+      <x:c r="C23" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="46" customHeight="1">
       <x:c r="A24" s="4" t="str">
@@ -605,8 +687,12 @@
       <x:c r="B24" s="4" t="str">
         <x:v>https://github.com/ckan/ckan</x:v>
       </x:c>
-      <x:c r="C24" s="4"/>
-      <x:c r="D24" s="4"/>
+      <x:c r="C24" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="46" customHeight="1">
       <x:c r="A25" s="4" t="str">
@@ -615,8 +701,12 @@
       <x:c r="B25" s="4" t="str">
         <x:v>https://github.com/copilot-emacs/copilot.el</x:v>
       </x:c>
-      <x:c r="C25" s="4"/>
-      <x:c r="D25" s="4"/>
+      <x:c r="C25" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="46" customHeight="1">
       <x:c r="A26" s="4" t="str">
@@ -625,8 +715,12 @@
       <x:c r="B26" s="4" t="str">
         <x:v>https://github.com/crate/crate</x:v>
       </x:c>
-      <x:c r="C26" s="4"/>
-      <x:c r="D26" s="4"/>
+      <x:c r="C26" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="46" customHeight="1">
       <x:c r="A27" s="4" t="str">
@@ -635,8 +729,12 @@
       <x:c r="B27" s="4" t="str">
         <x:v>https://github.com/cypress-io/github-action</x:v>
       </x:c>
-      <x:c r="C27" s="4"/>
-      <x:c r="D27" s="4"/>
+      <x:c r="C27" s="4" t="str">
+        <x:v>outro</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="46" customHeight="1">
       <x:c r="A28" s="4" t="str">
@@ -645,8 +743,12 @@
       <x:c r="B28" s="4" t="str">
         <x:v>https://github.com/deer-flow/llm-space</x:v>
       </x:c>
-      <x:c r="C28" s="4"/>
-      <x:c r="D28" s="4"/>
+      <x:c r="C28" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="46" customHeight="1">
       <x:c r="A29" s="4" t="str">
@@ -655,8 +757,12 @@
       <x:c r="B29" s="4" t="str">
         <x:v>https://github.com/googleads/googleads-mobile-ios-examples</x:v>
       </x:c>
-      <x:c r="C29" s="4"/>
-      <x:c r="D29" s="4"/>
+      <x:c r="C29" s="4" t="str">
+        <x:v>outro</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="46" customHeight="1">
       <x:c r="A30" s="4" t="str">
@@ -665,8 +771,12 @@
       <x:c r="B30" s="4" t="str">
         <x:v>https://github.com/guhcostan/mac-cleaner-cli</x:v>
       </x:c>
-      <x:c r="C30" s="4"/>
-      <x:c r="D30" s="4"/>
+      <x:c r="C30" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="46" customHeight="1">
       <x:c r="A31" s="4" t="str">
@@ -675,8 +785,12 @@
       <x:c r="B31" s="4" t="str">
         <x:v>https://github.com/hardbeat920/monocode</x:v>
       </x:c>
-      <x:c r="C31" s="4"/>
-      <x:c r="D31" s="4"/>
+      <x:c r="C31" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="46" customHeight="1">
       <x:c r="A32" s="4" t="str">
@@ -685,8 +799,12 @@
       <x:c r="B32" s="4" t="str">
         <x:v>https://github.com/htmlhint/HTMLHint</x:v>
       </x:c>
-      <x:c r="C32" s="4"/>
-      <x:c r="D32" s="4"/>
+      <x:c r="C32" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="46" customHeight="1">
       <x:c r="A33" s="4" t="str">
@@ -695,8 +813,12 @@
       <x:c r="B33" s="4" t="str">
         <x:v>https://github.com/jenkinsci/docker</x:v>
       </x:c>
-      <x:c r="C33" s="4"/>
-      <x:c r="D33" s="4"/>
+      <x:c r="C33" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="46" customHeight="1">
       <x:c r="A34" s="4" t="str">
@@ -705,8 +827,12 @@
       <x:c r="B34" s="4" t="str">
         <x:v>https://github.com/jhomlala/betterplayer</x:v>
       </x:c>
-      <x:c r="C34" s="4"/>
-      <x:c r="D34" s="4"/>
+      <x:c r="C34" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D34" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="46" customHeight="1">
       <x:c r="A35" s="4" t="str">
@@ -715,8 +841,12 @@
       <x:c r="B35" s="4" t="str">
         <x:v>https://github.com/kubeshop/testkube</x:v>
       </x:c>
-      <x:c r="C35" s="4"/>
-      <x:c r="D35" s="4"/>
+      <x:c r="C35" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="46" customHeight="1">
       <x:c r="A36" s="4" t="str">
@@ -725,8 +855,12 @@
       <x:c r="B36" s="4" t="str">
         <x:v>https://github.com/liveblocks/liveblocks</x:v>
       </x:c>
-      <x:c r="C36" s="4"/>
-      <x:c r="D36" s="4"/>
+      <x:c r="C36" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D36" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="46" customHeight="1">
       <x:c r="A37" s="4" t="str">
@@ -735,8 +869,12 @@
       <x:c r="B37" s="4" t="str">
         <x:v>https://github.com/loro-dev/loro</x:v>
       </x:c>
-      <x:c r="C37" s="4"/>
-      <x:c r="D37" s="4"/>
+      <x:c r="C37" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="46" customHeight="1">
       <x:c r="A38" s="4" t="str">
@@ -745,8 +883,12 @@
       <x:c r="B38" s="4" t="str">
         <x:v>https://github.com/microsoft/mcp</x:v>
       </x:c>
-      <x:c r="C38" s="4"/>
-      <x:c r="D38" s="4"/>
+      <x:c r="C38" s="4" t="str">
+        <x:v>outro</x:v>
+      </x:c>
+      <x:c r="D38" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="46" customHeight="1">
       <x:c r="A39" s="4" t="str">
@@ -755,8 +897,12 @@
       <x:c r="B39" s="4" t="str">
         <x:v>https://github.com/mivano/azure-cost-cli</x:v>
       </x:c>
-      <x:c r="C39" s="4"/>
-      <x:c r="D39" s="4"/>
+      <x:c r="C39" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="46" customHeight="1">
       <x:c r="A40" s="4" t="str">
@@ -765,8 +911,12 @@
       <x:c r="B40" s="4" t="str">
         <x:v>https://github.com/mozilla/pontoon</x:v>
       </x:c>
-      <x:c r="C40" s="4"/>
-      <x:c r="D40" s="4"/>
+      <x:c r="C40" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D40" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="46" customHeight="1">
       <x:c r="A41" s="4" t="str">
@@ -775,8 +925,12 @@
       <x:c r="B41" s="4" t="str">
         <x:v>https://github.com/node-opcua/node-opcua</x:v>
       </x:c>
-      <x:c r="C41" s="4"/>
-      <x:c r="D41" s="4"/>
+      <x:c r="C41" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="46" customHeight="1">
       <x:c r="A42" s="4" t="str">
@@ -785,8 +939,12 @@
       <x:c r="B42" s="4" t="str">
         <x:v>https://github.com/odygrd/quill</x:v>
       </x:c>
-      <x:c r="C42" s="4"/>
-      <x:c r="D42" s="4"/>
+      <x:c r="C42" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D42" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="46" customHeight="1">
       <x:c r="A43" s="4" t="str">
@@ -795,8 +953,12 @@
       <x:c r="B43" s="4" t="str">
         <x:v>https://github.com/open-logic/open-logic</x:v>
       </x:c>
-      <x:c r="C43" s="4"/>
-      <x:c r="D43" s="4"/>
+      <x:c r="C43" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="46" customHeight="1">
       <x:c r="A44" s="4" t="str">
@@ -805,8 +967,12 @@
       <x:c r="B44" s="4" t="str">
         <x:v>https://github.com/opengeos/geoai</x:v>
       </x:c>
-      <x:c r="C44" s="4"/>
-      <x:c r="D44" s="4"/>
+      <x:c r="C44" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D44" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="46" customHeight="1">
       <x:c r="A45" s="4" t="str">
@@ -815,8 +981,12 @@
       <x:c r="B45" s="4" t="str">
         <x:v>https://github.com/pgjdbc/pgjdbc</x:v>
       </x:c>
-      <x:c r="C45" s="4"/>
-      <x:c r="D45" s="4"/>
+      <x:c r="C45" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D45" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="46" customHeight="1">
       <x:c r="A46" s="4" t="str">
@@ -825,8 +995,12 @@
       <x:c r="B46" s="4" t="str">
         <x:v>https://github.com/prebid/Prebid.js</x:v>
       </x:c>
-      <x:c r="C46" s="4"/>
-      <x:c r="D46" s="4"/>
+      <x:c r="C46" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D46" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="46" customHeight="1">
       <x:c r="A47" s="4" t="str">
@@ -835,8 +1009,12 @@
       <x:c r="B47" s="4" t="str">
         <x:v>https://github.com/project-zot/zot</x:v>
       </x:c>
-      <x:c r="C47" s="4"/>
-      <x:c r="D47" s="4"/>
+      <x:c r="C47" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D47" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="46" customHeight="1">
       <x:c r="A48" s="4" t="str">
@@ -845,8 +1023,12 @@
       <x:c r="B48" s="4" t="str">
         <x:v>https://github.com/puemos/craftplan</x:v>
       </x:c>
-      <x:c r="C48" s="4"/>
-      <x:c r="D48" s="4"/>
+      <x:c r="C48" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D48" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="46" customHeight="1">
       <x:c r="A49" s="4" t="str">
@@ -855,8 +1037,12 @@
       <x:c r="B49" s="4" t="str">
         <x:v>https://github.com/puma/puma</x:v>
       </x:c>
-      <x:c r="C49" s="4"/>
-      <x:c r="D49" s="4"/>
+      <x:c r="C49" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D49" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="46" customHeight="1">
       <x:c r="A50" s="4" t="str">
@@ -865,8 +1051,12 @@
       <x:c r="B50" s="4" t="str">
         <x:v>https://github.com/pymc-labs/pymc-marketing</x:v>
       </x:c>
-      <x:c r="C50" s="4"/>
-      <x:c r="D50" s="4"/>
+      <x:c r="C50" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D50" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="46" customHeight="1">
       <x:c r="A51" s="4" t="str">
@@ -875,8 +1065,12 @@
       <x:c r="B51" s="4" t="str">
         <x:v>https://github.com/qiutongxue/oba-live-tool</x:v>
       </x:c>
-      <x:c r="C51" s="4"/>
-      <x:c r="D51" s="4"/>
+      <x:c r="C51" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D51" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="46" customHeight="1">
       <x:c r="A52" s="4" t="str">
@@ -885,8 +1079,12 @@
       <x:c r="B52" s="4" t="str">
         <x:v>https://github.com/qiz029/dscode</x:v>
       </x:c>
-      <x:c r="C52" s="4"/>
-      <x:c r="D52" s="4"/>
+      <x:c r="C52" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D52" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="46" customHeight="1">
       <x:c r="A53" s="4" t="str">
@@ -895,8 +1093,12 @@
       <x:c r="B53" s="4" t="str">
         <x:v>https://github.com/remorses/playwriter</x:v>
       </x:c>
-      <x:c r="C53" s="4"/>
-      <x:c r="D53" s="4"/>
+      <x:c r="C53" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D53" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="46" customHeight="1">
       <x:c r="A54" s="4" t="str">
@@ -905,8 +1107,12 @@
       <x:c r="B54" s="4" t="str">
         <x:v>https://github.com/rhysd/actionlint</x:v>
       </x:c>
-      <x:c r="C54" s="4"/>
-      <x:c r="D54" s="4"/>
+      <x:c r="C54" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D54" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="46" customHeight="1">
       <x:c r="A55" s="4" t="str">
@@ -915,8 +1121,12 @@
       <x:c r="B55" s="4" t="str">
         <x:v>https://github.com/superdoc/docx-editor</x:v>
       </x:c>
-      <x:c r="C55" s="4"/>
-      <x:c r="D55" s="4"/>
+      <x:c r="C55" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D55" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="46" customHeight="1">
       <x:c r="A56" s="4" t="str">
@@ -925,8 +1135,12 @@
       <x:c r="B56" s="4" t="str">
         <x:v>https://github.com/unicode-org/icu4x</x:v>
       </x:c>
-      <x:c r="C56" s="4"/>
-      <x:c r="D56" s="4"/>
+      <x:c r="C56" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D56" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="46" customHeight="1">
       <x:c r="A57" s="4" t="str">
@@ -935,8 +1149,12 @@
       <x:c r="B57" s="4" t="str">
         <x:v>https://github.com/utkuozdemir/pv-migrate</x:v>
       </x:c>
-      <x:c r="C57" s="4"/>
-      <x:c r="D57" s="4"/>
+      <x:c r="C57" s="4" t="str">
+        <x:v>ferramenta CLI</x:v>
+      </x:c>
+      <x:c r="D57" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="46" customHeight="1">
       <x:c r="A58" s="4" t="str">
@@ -945,8 +1163,12 @@
       <x:c r="B58" s="4" t="str">
         <x:v>https://github.com/vergecurrency/verge</x:v>
       </x:c>
-      <x:c r="C58" s="4"/>
-      <x:c r="D58" s="4"/>
+      <x:c r="C58" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D58" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="46" customHeight="1">
       <x:c r="A59" s="4" t="str">
@@ -955,8 +1177,12 @@
       <x:c r="B59" s="4" t="str">
         <x:v>https://github.com/vllm-project/llm-compressor</x:v>
       </x:c>
-      <x:c r="C59" s="4"/>
-      <x:c r="D59" s="4"/>
+      <x:c r="C59" s="4" t="str">
+        <x:v>biblioteca/framework</x:v>
+      </x:c>
+      <x:c r="D59" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="46" customHeight="1">
       <x:c r="A60" s="4" t="str">
@@ -965,8 +1191,12 @@
       <x:c r="B60" s="4" t="str">
         <x:v>https://github.com/yhan-sun/p2wlan</x:v>
       </x:c>
-      <x:c r="C60" s="4"/>
-      <x:c r="D60" s="4"/>
+      <x:c r="C60" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D60" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="46" customHeight="1">
       <x:c r="A61" s="4" t="str">
@@ -975,8 +1205,12 @@
       <x:c r="B61" s="4" t="str">
         <x:v>https://github.com/zerx-lab/FluxDown</x:v>
       </x:c>
-      <x:c r="C61" s="4"/>
-      <x:c r="D61" s="4"/>
+      <x:c r="C61" s="4" t="str">
+        <x:v>aplicação/serviço</x:v>
+      </x:c>
+      <x:c r="D61" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -1039,7 +1273,9 @@
       <x:c r="E2" s="4" t="str">
         <x:v>https://github.com/Azure/AKS/compare/2025-09-21...2025-10-12</x:v>
       </x:c>
-      <x:c r="F2" s="4"/>
+      <x:c r="F2" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="46" customHeight="1">
       <x:c r="A3" s="4" t="str">
@@ -1057,7 +1293,9 @@
       <x:c r="E3" s="4" t="str">
         <x:v>https://github.com/Azure/AKS/compare/2026-04-02...2026-04-28</x:v>
       </x:c>
-      <x:c r="F3" s="4"/>
+      <x:c r="F3" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="46" customHeight="1">
       <x:c r="A4" s="4" t="str">
@@ -1075,7 +1313,9 @@
       <x:c r="E4" s="4" t="str">
         <x:v>https://github.com/Azure/AKS/compare/2026-06-19...2026-07-17</x:v>
       </x:c>
-      <x:c r="F4" s="4"/>
+      <x:c r="F4" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="46" customHeight="1">
       <x:c r="A5" s="4" t="str">
@@ -1093,7 +1333,9 @@
       <x:c r="E5" s="4" t="str">
         <x:v>https://github.com/Azure/AKS/compare/2026-07-17...2026-08-07</x:v>
       </x:c>
-      <x:c r="F5" s="4"/>
+      <x:c r="F5" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="4" t="str">
@@ -1111,7 +1353,9 @@
       <x:c r="E6" s="4" t="str">
         <x:v>https://github.com/Azure/AKS/compare/2026-08-07...AppNet-2026-08-19</x:v>
       </x:c>
-      <x:c r="F6" s="4"/>
+      <x:c r="F6" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
       <x:c r="A7" s="4" t="str">
@@ -1127,7 +1371,9 @@
         <x:v>https://github.com/Chorus-AIDLC/Chorus/releases/tag/v0.1.0</x:v>
       </x:c>
       <x:c r="E7" s="4"/>
-      <x:c r="F7" s="4"/>
+      <x:c r="F7" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
       <x:c r="A8" s="4" t="str">
@@ -1145,7 +1391,9 @@
       <x:c r="E8" s="4" t="str">
         <x:v>https://github.com/Chorus-AIDLC/Chorus/compare/v0.4.0...v0.4.1</x:v>
       </x:c>
-      <x:c r="F8" s="4"/>
+      <x:c r="F8" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
       <x:c r="A9" s="4" t="str">
@@ -1163,7 +1411,9 @@
       <x:c r="E9" s="4" t="str">
         <x:v>https://github.com/Chorus-AIDLC/Chorus/compare/v0.6.3...v0.6.4</x:v>
       </x:c>
-      <x:c r="F9" s="4"/>
+      <x:c r="F9" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
       <x:c r="A10" s="4" t="str">
@@ -1181,7 +1431,9 @@
       <x:c r="E10" s="4" t="str">
         <x:v>https://github.com/Chorus-AIDLC/Chorus/compare/v0.12.0...v0.12.1</x:v>
       </x:c>
-      <x:c r="F10" s="4"/>
+      <x:c r="F10" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
       <x:c r="A11" s="4" t="str">
@@ -1199,7 +1451,9 @@
       <x:c r="E11" s="4" t="str">
         <x:v>https://github.com/Chorus-AIDLC/Chorus/compare/v0.13.2...v0.14.0</x:v>
       </x:c>
-      <x:c r="F11" s="4"/>
+      <x:c r="F11" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
       <x:c r="A12" s="4" t="str">
@@ -1215,7 +1469,9 @@
         <x:v>https://github.com/Darkatse/TauriTavern/releases/tag/v1.0.0</x:v>
       </x:c>
       <x:c r="E12" s="4"/>
-      <x:c r="F12" s="4"/>
+      <x:c r="F12" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
       <x:c r="A13" s="4" t="str">
@@ -1233,7 +1489,9 @@
       <x:c r="E13" s="4" t="str">
         <x:v>https://github.com/Darkatse/TauriTavern/compare/v1.3.0...v1.4.0</x:v>
       </x:c>
-      <x:c r="F13" s="4"/>
+      <x:c r="F13" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
       <x:c r="A14" s="4" t="str">
@@ -1251,7 +1509,9 @@
       <x:c r="E14" s="4" t="str">
         <x:v>https://github.com/Darkatse/TauriTavern/compare/v1.4.2...v1.5.0</x:v>
       </x:c>
-      <x:c r="F14" s="4"/>
+      <x:c r="F14" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
       <x:c r="A15" s="4" t="str">
@@ -1269,7 +1529,9 @@
       <x:c r="E15" s="4" t="str">
         <x:v>https://github.com/Darkatse/TauriTavern/compare/v1.6.0...v1.6.1</x:v>
       </x:c>
-      <x:c r="F15" s="4"/>
+      <x:c r="F15" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
       <x:c r="A16" s="4" t="str">
@@ -1287,7 +1549,9 @@
       <x:c r="E16" s="4" t="str">
         <x:v>https://github.com/Darkatse/TauriTavern/compare/v2.1.1...v2.2.0</x:v>
       </x:c>
-      <x:c r="F16" s="4"/>
+      <x:c r="F16" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
       <x:c r="A17" s="4" t="str">
@@ -1305,7 +1569,9 @@
       <x:c r="E17" s="4" t="str">
         <x:v>https://github.com/GetStream/stream-chat-flutter/compare/v9.17.0...v9.18.0</x:v>
       </x:c>
-      <x:c r="F17" s="4"/>
+      <x:c r="F17" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
       <x:c r="A18" s="4" t="str">
@@ -1323,7 +1589,9 @@
       <x:c r="E18" s="4" t="str">
         <x:v>https://github.com/GetStream/stream-chat-flutter/compare/v9.18.0...v9.19.0</x:v>
       </x:c>
-      <x:c r="F18" s="4"/>
+      <x:c r="F18" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="46" customHeight="1">
       <x:c r="A19" s="4" t="str">
@@ -1341,7 +1609,9 @@
       <x:c r="E19" s="4" t="str">
         <x:v>https://github.com/GetStream/stream-chat-flutter/compare/v9.25.0...v10.0.1</x:v>
       </x:c>
-      <x:c r="F19" s="4"/>
+      <x:c r="F19" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="46" customHeight="1">
       <x:c r="A20" s="4" t="str">
@@ -1359,7 +1629,9 @@
       <x:c r="E20" s="4" t="str">
         <x:v>https://github.com/GetStream/stream-chat-flutter/compare/v9.28.0...v10.4.0</x:v>
       </x:c>
-      <x:c r="F20" s="4"/>
+      <x:c r="F20" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="46" customHeight="1">
       <x:c r="A21" s="4" t="str">
@@ -1377,7 +1649,9 @@
       <x:c r="E21" s="4" t="str">
         <x:v>https://github.com/GetStream/stream-chat-flutter/compare/v9.29.0...v9.30.0</x:v>
       </x:c>
-      <x:c r="F21" s="4"/>
+      <x:c r="F21" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="46" customHeight="1">
       <x:c r="A22" s="4" t="str">
@@ -1393,7 +1667,9 @@
         <x:v>https://github.com/MGdaasLab/WHartTest/releases/tag/v1.2.0</x:v>
       </x:c>
       <x:c r="E22" s="4"/>
-      <x:c r="F22" s="4"/>
+      <x:c r="F22" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="46" customHeight="1">
       <x:c r="A23" s="4" t="str">
@@ -1411,7 +1687,9 @@
       <x:c r="E23" s="4" t="str">
         <x:v>https://github.com/MGdaasLab/WHartTest/compare/v1.2.0...v1.3.0</x:v>
       </x:c>
-      <x:c r="F23" s="4"/>
+      <x:c r="F23" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="46" customHeight="1">
       <x:c r="A24" s="4" t="str">
@@ -1429,7 +1707,9 @@
       <x:c r="E24" s="4" t="str">
         <x:v>https://github.com/MGdaasLab/WHartTest/compare/v2.2.0...v2.3.0</x:v>
       </x:c>
-      <x:c r="F24" s="4"/>
+      <x:c r="F24" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="46" customHeight="1">
       <x:c r="A25" s="4" t="str">
@@ -1447,7 +1727,9 @@
       <x:c r="E25" s="4" t="str">
         <x:v>https://github.com/MGdaasLab/WHartTest/compare/v2.5.0...v2.5.1</x:v>
       </x:c>
-      <x:c r="F25" s="4"/>
+      <x:c r="F25" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="46" customHeight="1">
       <x:c r="A26" s="4" t="str">
@@ -1465,7 +1747,9 @@
       <x:c r="E26" s="4" t="str">
         <x:v>https://github.com/MGdaasLab/WHartTest/compare/v2.6.0...v2.7.0</x:v>
       </x:c>
-      <x:c r="F26" s="4"/>
+      <x:c r="F26" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="46" customHeight="1">
       <x:c r="A27" s="4" t="str">
@@ -1483,7 +1767,9 @@
       <x:c r="E27" s="4" t="str">
         <x:v>https://github.com/MaikuB/flutter_local_notifications/compare/flutter_local_notifications-v19.4.2...flutter_local_notifications-v19.5.0</x:v>
       </x:c>
-      <x:c r="F27" s="4"/>
+      <x:c r="F27" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="46" customHeight="1">
       <x:c r="A28" s="4" t="str">
@@ -1501,7 +1787,9 @@
       <x:c r="E28" s="4" t="str">
         <x:v>https://github.com/MaikuB/flutter_local_notifications/compare/flutter_local_notifications-v19.5.0...flutter_local_notifications-v20.0.0</x:v>
       </x:c>
-      <x:c r="F28" s="4"/>
+      <x:c r="F28" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="46" customHeight="1">
       <x:c r="A29" s="4" t="str">
@@ -1519,7 +1807,9 @@
       <x:c r="E29" s="4" t="str">
         <x:v>https://github.com/MaikuB/flutter_local_notifications/compare/flutter_local_notifications-v22.0.0...flutter_local_notifications-v22.0.1</x:v>
       </x:c>
-      <x:c r="F29" s="4"/>
+      <x:c r="F29" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="46" customHeight="1">
       <x:c r="A30" s="4" t="str">
@@ -1537,7 +1827,9 @@
       <x:c r="E30" s="4" t="str">
         <x:v>https://github.com/MaikuB/flutter_local_notifications/compare/flutter_local_notifications-v22.1.0...flutter_local_notifications-v22.2.0</x:v>
       </x:c>
-      <x:c r="F30" s="4"/>
+      <x:c r="F30" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="46" customHeight="1">
       <x:c r="A31" s="4" t="str">
@@ -1555,7 +1847,9 @@
       <x:c r="E31" s="4" t="str">
         <x:v>https://github.com/MaikuB/flutter_local_notifications/compare/flutter_local_notifications-v22.2.0...flutter_local_notifications-v22.3.0</x:v>
       </x:c>
-      <x:c r="F31" s="4"/>
+      <x:c r="F31" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="46" customHeight="1">
       <x:c r="A32" s="4" t="str">
@@ -1573,7 +1867,9 @@
       <x:c r="E32" s="4" t="str">
         <x:v>https://github.com/NVIDIA-NeMo/Guardrails/compare/v0.16.0...v0.17.0</x:v>
       </x:c>
-      <x:c r="F32" s="4"/>
+      <x:c r="F32" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="46" customHeight="1">
       <x:c r="A33" s="4" t="str">
@@ -1591,7 +1887,9 @@
       <x:c r="E33" s="4" t="str">
         <x:v>https://github.com/NVIDIA-NeMo/Guardrails/compare/v0.17.0...v0.18.0</x:v>
       </x:c>
-      <x:c r="F33" s="4"/>
+      <x:c r="F33" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="46" customHeight="1">
       <x:c r="A34" s="4" t="str">
@@ -1609,7 +1907,9 @@
       <x:c r="E34" s="4" t="str">
         <x:v>https://github.com/NVIDIA-NeMo/Guardrails/compare/v0.21.0...v0.22.0</x:v>
       </x:c>
-      <x:c r="F34" s="4"/>
+      <x:c r="F34" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="46" customHeight="1">
       <x:c r="A35" s="4" t="str">
@@ -1627,7 +1927,9 @@
       <x:c r="E35" s="4" t="str">
         <x:v>https://github.com/NVIDIA-NeMo/Guardrails/compare/v0.23.0...v0.24.0</x:v>
       </x:c>
-      <x:c r="F35" s="4"/>
+      <x:c r="F35" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="46" customHeight="1">
       <x:c r="A36" s="4" t="str">
@@ -1645,7 +1947,9 @@
       <x:c r="E36" s="4" t="str">
         <x:v>https://github.com/NVIDIA-NeMo/Guardrails/compare/v0.24.0...v0.24.1</x:v>
       </x:c>
-      <x:c r="F36" s="4"/>
+      <x:c r="F36" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="46" customHeight="1">
       <x:c r="A37" s="4" t="str">
@@ -1663,7 +1967,9 @@
       <x:c r="E37" s="4" t="str">
         <x:v>https://github.com/StuffAnThings/qbit_manage/compare/v4.6.3...v4.6.4</x:v>
       </x:c>
-      <x:c r="F37" s="4"/>
+      <x:c r="F37" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="46" customHeight="1">
       <x:c r="A38" s="4" t="str">
@@ -1681,7 +1987,9 @@
       <x:c r="E38" s="4" t="str">
         <x:v>https://github.com/StuffAnThings/qbit_manage/compare/v4.7.1...v4.8.0</x:v>
       </x:c>
-      <x:c r="F38" s="4"/>
+      <x:c r="F38" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="46" customHeight="1">
       <x:c r="A39" s="4" t="str">
@@ -1699,7 +2007,9 @@
       <x:c r="E39" s="4" t="str">
         <x:v>https://github.com/StuffAnThings/qbit_manage/compare/v4.9.1...v4.10.0</x:v>
       </x:c>
-      <x:c r="F39" s="4"/>
+      <x:c r="F39" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="46" customHeight="1">
       <x:c r="A40" s="4" t="str">
@@ -1717,7 +2027,9 @@
       <x:c r="E40" s="4" t="str">
         <x:v>https://github.com/StuffAnThings/qbit_manage/compare/v4.10.0...v4.11.0</x:v>
       </x:c>
-      <x:c r="F40" s="4"/>
+      <x:c r="F40" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="46" customHeight="1">
       <x:c r="A41" s="4" t="str">
@@ -1735,7 +2047,9 @@
       <x:c r="E41" s="4" t="str">
         <x:v>https://github.com/StuffAnThings/qbit_manage/compare/v4.11.0...v4.12.0</x:v>
       </x:c>
-      <x:c r="F41" s="4"/>
+      <x:c r="F41" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="46" customHeight="1">
       <x:c r="A42" s="4" t="str">
@@ -1753,7 +2067,9 @@
       <x:c r="E42" s="4" t="str">
         <x:v>https://github.com/Sync-in/server/compare/v1.6.0...v1.6.1</x:v>
       </x:c>
-      <x:c r="F42" s="4"/>
+      <x:c r="F42" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="46" customHeight="1">
       <x:c r="A43" s="4" t="str">
@@ -1771,7 +2087,9 @@
       <x:c r="E43" s="4" t="str">
         <x:v>https://github.com/Sync-in/server/compare/v1.10.0...v1.10.1</x:v>
       </x:c>
-      <x:c r="F43" s="4"/>
+      <x:c r="F43" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="46" customHeight="1">
       <x:c r="A44" s="4" t="str">
@@ -1789,7 +2107,9 @@
       <x:c r="E44" s="4" t="str">
         <x:v>https://github.com/Sync-in/server/compare/v1.10.1...v1.11.0</x:v>
       </x:c>
-      <x:c r="F44" s="4"/>
+      <x:c r="F44" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="46" customHeight="1">
       <x:c r="A45" s="4" t="str">
@@ -1807,7 +2127,9 @@
       <x:c r="E45" s="4" t="str">
         <x:v>https://github.com/Sync-in/server/compare/v2.3.0...v2.4.0</x:v>
       </x:c>
-      <x:c r="F45" s="4"/>
+      <x:c r="F45" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="46" customHeight="1">
       <x:c r="A46" s="4" t="str">
@@ -1825,7 +2147,9 @@
       <x:c r="E46" s="4" t="str">
         <x:v>https://github.com/Sync-in/server/compare/v2.4.1...v2.4.2</x:v>
       </x:c>
-      <x:c r="F46" s="4"/>
+      <x:c r="F46" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="46" customHeight="1">
       <x:c r="A47" s="4" t="str">
@@ -1843,7 +2167,9 @@
       <x:c r="E47" s="4" t="str">
         <x:v>https://github.com/TNG/ArchUnitNET/compare/0.12.3...0.13.0</x:v>
       </x:c>
-      <x:c r="F47" s="4"/>
+      <x:c r="F47" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="46" customHeight="1">
       <x:c r="A48" s="4" t="str">
@@ -1861,7 +2187,9 @@
       <x:c r="E48" s="4" t="str">
         <x:v>https://github.com/TNG/ArchUnitNET/compare/0.13.0...0.13.1</x:v>
       </x:c>
-      <x:c r="F48" s="4"/>
+      <x:c r="F48" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="46" customHeight="1">
       <x:c r="A49" s="4" t="str">
@@ -1879,7 +2207,9 @@
       <x:c r="E49" s="4" t="str">
         <x:v>https://github.com/TNG/ArchUnitNET/compare/0.13.1...0.13.2</x:v>
       </x:c>
-      <x:c r="F49" s="4"/>
+      <x:c r="F49" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="46" customHeight="1">
       <x:c r="A50" s="4" t="str">
@@ -1897,7 +2227,9 @@
       <x:c r="E50" s="4" t="str">
         <x:v>https://github.com/TNG/ArchUnitNET/compare/0.13.2...0.13.3</x:v>
       </x:c>
-      <x:c r="F50" s="4"/>
+      <x:c r="F50" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="46" customHeight="1">
       <x:c r="A51" s="4" t="str">
@@ -1915,7 +2247,9 @@
       <x:c r="E51" s="4" t="str">
         <x:v>https://github.com/TNG/ArchUnitNET/compare/0.13.3...0.13.4</x:v>
       </x:c>
-      <x:c r="F51" s="4"/>
+      <x:c r="F51" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="46" customHeight="1">
       <x:c r="A52" s="4" t="str">
@@ -1933,7 +2267,9 @@
       <x:c r="E52" s="4" t="str">
         <x:v>https://github.com/Ylianst/MeshCentral/compare/1.1.51...1.1.52</x:v>
       </x:c>
-      <x:c r="F52" s="4"/>
+      <x:c r="F52" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="46" customHeight="1">
       <x:c r="A53" s="4" t="str">
@@ -1951,7 +2287,9 @@
       <x:c r="E53" s="4" t="str">
         <x:v>https://github.com/Ylianst/MeshCentral/compare/1.1.52...1.1.53</x:v>
       </x:c>
-      <x:c r="F53" s="4"/>
+      <x:c r="F53" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="46" customHeight="1">
       <x:c r="A54" s="4" t="str">
@@ -1969,7 +2307,9 @@
       <x:c r="E54" s="4" t="str">
         <x:v>https://github.com/Ylianst/MeshCentral/compare/1.1.56...1.1.57</x:v>
       </x:c>
-      <x:c r="F54" s="4"/>
+      <x:c r="F54" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="46" customHeight="1">
       <x:c r="A55" s="4" t="str">
@@ -1987,7 +2327,9 @@
       <x:c r="E55" s="4" t="str">
         <x:v>https://github.com/Ylianst/MeshCentral/compare/1.2.3...1.2.4</x:v>
       </x:c>
-      <x:c r="F55" s="4"/>
+      <x:c r="F55" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="46" customHeight="1">
       <x:c r="A56" s="4" t="str">
@@ -2005,7 +2347,9 @@
       <x:c r="E56" s="4" t="str">
         <x:v>https://github.com/Ylianst/MeshCentral/compare/1.2.4...1.2.5</x:v>
       </x:c>
-      <x:c r="F56" s="4"/>
+      <x:c r="F56" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="46" customHeight="1">
       <x:c r="A57" s="4" t="str">
@@ -2023,7 +2367,9 @@
       <x:c r="E57" s="4" t="str">
         <x:v>https://github.com/actions/cache/compare/v3.5.0...v5.0.0</x:v>
       </x:c>
-      <x:c r="F57" s="4"/>
+      <x:c r="F57" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="46" customHeight="1">
       <x:c r="A58" s="4" t="str">
@@ -2041,7 +2387,9 @@
       <x:c r="E58" s="4" t="str">
         <x:v>https://github.com/actions/cache/compare/v5.0.0...v5.0.1</x:v>
       </x:c>
-      <x:c r="F58" s="4"/>
+      <x:c r="F58" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="46" customHeight="1">
       <x:c r="A59" s="4" t="str">
@@ -2059,7 +2407,9 @@
       <x:c r="E59" s="4" t="str">
         <x:v>https://github.com/actions/cache/compare/v5.0.4...v5.0.5</x:v>
       </x:c>
-      <x:c r="F59" s="4"/>
+      <x:c r="F59" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="46" customHeight="1">
       <x:c r="A60" s="4" t="str">
@@ -2077,7 +2427,9 @@
       <x:c r="E60" s="4" t="str">
         <x:v>https://github.com/actions/cache/compare/v6.0.0...v6.1.0</x:v>
       </x:c>
-      <x:c r="F60" s="4"/>
+      <x:c r="F60" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="46" customHeight="1">
       <x:c r="A61" s="4" t="str">
@@ -2095,7 +2447,9 @@
       <x:c r="E61" s="4" t="str">
         <x:v>https://github.com/actions/cache/compare/v6.1.0...v5.1.0</x:v>
       </x:c>
-      <x:c r="F61" s="4"/>
+      <x:c r="F61" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="46" customHeight="1">
       <x:c r="A62" s="4" t="str">
@@ -2113,7 +2467,9 @@
       <x:c r="E62" s="4" t="str">
         <x:v>https://github.com/agavra/tuicr/compare/v0.9.0...v0.10.0</x:v>
       </x:c>
-      <x:c r="F62" s="4"/>
+      <x:c r="F62" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="46" customHeight="1">
       <x:c r="A63" s="4" t="str">
@@ -2131,7 +2487,9 @@
       <x:c r="E63" s="4" t="str">
         <x:v>https://github.com/agavra/tuicr/compare/v0.12.0...v0.13.0</x:v>
       </x:c>
-      <x:c r="F63" s="4"/>
+      <x:c r="F63" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="46" customHeight="1">
       <x:c r="A64" s="4" t="str">
@@ -2149,7 +2507,9 @@
       <x:c r="E64" s="4" t="str">
         <x:v>https://github.com/agavra/tuicr/compare/v0.19.0...v0.19.1</x:v>
       </x:c>
-      <x:c r="F64" s="4"/>
+      <x:c r="F64" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="46" customHeight="1">
       <x:c r="A65" s="4" t="str">
@@ -2167,7 +2527,9 @@
       <x:c r="E65" s="4" t="str">
         <x:v>https://github.com/agavra/tuicr/compare/v0.22.0...v0.23.0</x:v>
       </x:c>
-      <x:c r="F65" s="4"/>
+      <x:c r="F65" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="46" customHeight="1">
       <x:c r="A66" s="4" t="str">
@@ -2185,7 +2547,9 @@
       <x:c r="E66" s="4" t="str">
         <x:v>https://github.com/agavra/tuicr/compare/v0.26.0...v0.27.0</x:v>
       </x:c>
-      <x:c r="F66" s="4"/>
+      <x:c r="F66" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="46" customHeight="1">
       <x:c r="A67" s="4" t="str">
@@ -2203,7 +2567,9 @@
       <x:c r="E67" s="4" t="str">
         <x:v>https://github.com/apache/servicecomb-java-chassis/compare/2.8.27...2.9.2</x:v>
       </x:c>
-      <x:c r="F67" s="4"/>
+      <x:c r="F67" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="46" customHeight="1">
       <x:c r="A68" s="4" t="str">
@@ -2221,7 +2587,9 @@
       <x:c r="E68" s="4" t="str">
         <x:v>https://github.com/apache/servicecomb-java-chassis/compare/2.9.2...2.8.28</x:v>
       </x:c>
-      <x:c r="F68" s="4"/>
+      <x:c r="F68" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="46" customHeight="1">
       <x:c r="A69" s="4" t="str">
@@ -2239,7 +2607,9 @@
       <x:c r="E69" s="4" t="str">
         <x:v>https://github.com/apache/servicecomb-java-chassis/compare/2.8.28...2.8.29</x:v>
       </x:c>
-      <x:c r="F69" s="4"/>
+      <x:c r="F69" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="46" customHeight="1">
       <x:c r="A70" s="4" t="str">
@@ -2257,7 +2627,9 @@
       <x:c r="E70" s="4" t="str">
         <x:v>https://github.com/apache/servicecomb-java-chassis/compare/2.9.3...2.8.31</x:v>
       </x:c>
-      <x:c r="F70" s="4"/>
+      <x:c r="F70" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="46" customHeight="1">
       <x:c r="A71" s="4" t="str">
@@ -2275,7 +2647,9 @@
       <x:c r="E71" s="4" t="str">
         <x:v>https://github.com/apache/servicecomb-java-chassis/compare/2.9.4...2.9.5</x:v>
       </x:c>
-      <x:c r="F71" s="4"/>
+      <x:c r="F71" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="46" customHeight="1">
       <x:c r="A72" s="4" t="str">
@@ -2293,7 +2667,9 @@
       <x:c r="E72" s="4" t="str">
         <x:v>https://github.com/apify/fingerprint-suite/compare/v2.1.73...v2.1.74</x:v>
       </x:c>
-      <x:c r="F72" s="4"/>
+      <x:c r="F72" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="46" customHeight="1">
       <x:c r="A73" s="4" t="str">
@@ -2311,7 +2687,9 @@
       <x:c r="E73" s="4" t="str">
         <x:v>https://github.com/apify/fingerprint-suite/compare/v2.1.78...v2.1.79</x:v>
       </x:c>
-      <x:c r="F73" s="4"/>
+      <x:c r="F73" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="46" customHeight="1">
       <x:c r="A74" s="4" t="str">
@@ -2329,7 +2707,9 @@
       <x:c r="E74" s="4" t="str">
         <x:v>https://github.com/apify/fingerprint-suite/compare/v2.1.82...v2.1.83</x:v>
       </x:c>
-      <x:c r="F74" s="4"/>
+      <x:c r="F74" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="46" customHeight="1">
       <x:c r="A75" s="4" t="str">
@@ -2347,7 +2727,9 @@
       <x:c r="E75" s="4" t="str">
         <x:v>https://github.com/apify/fingerprint-suite/compare/v2.1.85...v2.1.86</x:v>
       </x:c>
-      <x:c r="F75" s="4"/>
+      <x:c r="F75" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="46" customHeight="1">
       <x:c r="A76" s="4" t="str">
@@ -2365,7 +2747,9 @@
       <x:c r="E76" s="4" t="str">
         <x:v>https://github.com/apify/fingerprint-suite/compare/v2.1.86...v2.1.87</x:v>
       </x:c>
-      <x:c r="F76" s="4"/>
+      <x:c r="F76" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="46" customHeight="1">
       <x:c r="A77" s="4" t="str">
@@ -2383,7 +2767,9 @@
       <x:c r="E77" s="4" t="str">
         <x:v>https://github.com/ardatan/graphql-tools/compare/release-1758568993779...release-1761833018921</x:v>
       </x:c>
-      <x:c r="F77" s="4"/>
+      <x:c r="F77" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="46" customHeight="1">
       <x:c r="A78" s="4" t="str">
@@ -2401,7 +2787,9 @@
       <x:c r="E78" s="4" t="str">
         <x:v>https://github.com/ardatan/graphql-tools/compare/release-1761833018921...release-1762270964217</x:v>
       </x:c>
-      <x:c r="F78" s="4"/>
+      <x:c r="F78" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="46" customHeight="1">
       <x:c r="A79" s="4" t="str">
@@ -2419,7 +2807,9 @@
       <x:c r="E79" s="4" t="str">
         <x:v>https://github.com/ardatan/graphql-tools/compare/release-1762898070675...release-1762942062826</x:v>
       </x:c>
-      <x:c r="F79" s="4"/>
+      <x:c r="F79" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="46" customHeight="1">
       <x:c r="A80" s="4" t="str">
@@ -2437,7 +2827,9 @@
       <x:c r="E80" s="4" t="str">
         <x:v>https://github.com/ardatan/graphql-tools/compare/release-1763693142685...release-1764324313752</x:v>
       </x:c>
-      <x:c r="F80" s="4"/>
+      <x:c r="F80" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="46" customHeight="1">
       <x:c r="A81" s="4" t="str">
@@ -2455,7 +2847,9 @@
       <x:c r="E81" s="4" t="str">
         <x:v>https://github.com/ardatan/graphql-tools/compare/release-1772723897561...release-1772725596254</x:v>
       </x:c>
-      <x:c r="F81" s="4"/>
+      <x:c r="F81" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="46" customHeight="1">
       <x:c r="A82" s="4" t="str">
@@ -2473,7 +2867,9 @@
       <x:c r="E82" s="4" t="str">
         <x:v>https://github.com/ariebovenberg/whenever/compare/0.9.2...0.9.3</x:v>
       </x:c>
-      <x:c r="F82" s="4"/>
+      <x:c r="F82" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="46" customHeight="1">
       <x:c r="A83" s="4" t="str">
@@ -2491,7 +2887,9 @@
       <x:c r="E83" s="4" t="str">
         <x:v>https://github.com/ariebovenberg/whenever/compare/0.9.3...0.8.10</x:v>
       </x:c>
-      <x:c r="F83" s="4"/>
+      <x:c r="F83" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="46" customHeight="1">
       <x:c r="A84" s="4" t="str">
@@ -2509,7 +2907,9 @@
       <x:c r="E84" s="4" t="str">
         <x:v>https://github.com/ariebovenberg/whenever/compare/0.10.0...0.10.1</x:v>
       </x:c>
-      <x:c r="F84" s="4"/>
+      <x:c r="F84" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="46" customHeight="1">
       <x:c r="A85" s="4" t="str">
@@ -2527,7 +2927,9 @@
       <x:c r="E85" s="4" t="str">
         <x:v>https://github.com/ariebovenberg/whenever/compare/0.10.2...0.10.3</x:v>
       </x:c>
-      <x:c r="F85" s="4"/>
+      <x:c r="F85" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="46" customHeight="1">
       <x:c r="A86" s="4" t="str">
@@ -2545,7 +2947,9 @@
       <x:c r="E86" s="4" t="str">
         <x:v>https://github.com/ariebovenberg/whenever/compare/0.10.3...0.10.4</x:v>
       </x:c>
-      <x:c r="F86" s="4"/>
+      <x:c r="F86" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="46" customHeight="1">
       <x:c r="A87" s="4" t="str">
@@ -2563,7 +2967,9 @@
       <x:c r="E87" s="4" t="str">
         <x:v>https://github.com/arkime/arkime/compare/v5.8.0...v5.8.1</x:v>
       </x:c>
-      <x:c r="F87" s="4"/>
+      <x:c r="F87" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="46" customHeight="1">
       <x:c r="A88" s="4" t="str">
@@ -2581,7 +2987,9 @@
       <x:c r="E88" s="4" t="str">
         <x:v>https://github.com/arkime/arkime/compare/v6.0.1...v6.1.0</x:v>
       </x:c>
-      <x:c r="F88" s="4"/>
+      <x:c r="F88" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="46" customHeight="1">
       <x:c r="A89" s="4" t="str">
@@ -2599,7 +3007,9 @@
       <x:c r="E89" s="4" t="str">
         <x:v>https://github.com/arkime/arkime/compare/v6.3.1...v6.4.0</x:v>
       </x:c>
-      <x:c r="F89" s="4"/>
+      <x:c r="F89" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="46" customHeight="1">
       <x:c r="A90" s="4" t="str">
@@ -2617,7 +3027,9 @@
       <x:c r="E90" s="4" t="str">
         <x:v>https://github.com/arkime/arkime/compare/v6.5.0...v6.6.0</x:v>
       </x:c>
-      <x:c r="F90" s="4"/>
+      <x:c r="F90" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="46" customHeight="1">
       <x:c r="A91" s="4" t="str">
@@ -2635,7 +3047,9 @@
       <x:c r="E91" s="4" t="str">
         <x:v>https://github.com/arkime/arkime/compare/v6.6.0...v6.7.0</x:v>
       </x:c>
-      <x:c r="F91" s="4"/>
+      <x:c r="F91" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="46" customHeight="1">
       <x:c r="A92" s="4" t="str">
@@ -2653,7 +3067,9 @@
       <x:c r="E92" s="4" t="str">
         <x:v>https://github.com/borgbase/vorta/compare/v0.10.3...v0.11.0</x:v>
       </x:c>
-      <x:c r="F92" s="4"/>
+      <x:c r="F92" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="46" customHeight="1">
       <x:c r="A93" s="4" t="str">
@@ -2671,7 +3087,9 @@
       <x:c r="E93" s="4" t="str">
         <x:v>https://github.com/borgbase/vorta/compare/v0.11.0...v0.11.1</x:v>
       </x:c>
-      <x:c r="F93" s="4"/>
+      <x:c r="F93" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="46" customHeight="1">
       <x:c r="A94" s="4" t="str">
@@ -2689,7 +3107,9 @@
       <x:c r="E94" s="4" t="str">
         <x:v>https://github.com/borgbase/vorta/compare/v0.11.1...v0.11.2</x:v>
       </x:c>
-      <x:c r="F94" s="4"/>
+      <x:c r="F94" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="46" customHeight="1">
       <x:c r="A95" s="4" t="str">
@@ -2707,7 +3127,9 @@
       <x:c r="E95" s="4" t="str">
         <x:v>https://github.com/borgbase/vorta/compare/v0.11.3...v0.11.4</x:v>
       </x:c>
-      <x:c r="F95" s="4"/>
+      <x:c r="F95" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="46" customHeight="1">
       <x:c r="A96" s="4" t="str">
@@ -2725,7 +3147,9 @@
       <x:c r="E96" s="4" t="str">
         <x:v>https://github.com/borgbase/vorta/compare/v0.11.4...v0.11.5</x:v>
       </x:c>
-      <x:c r="F96" s="4"/>
+      <x:c r="F96" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" ht="46" customHeight="1">
       <x:c r="A97" s="4" t="str">
@@ -2743,7 +3167,9 @@
       <x:c r="E97" s="4" t="str">
         <x:v>https://github.com/bpg/terraform-provider-proxmox/compare/v0.87.0...v0.88.0</x:v>
       </x:c>
-      <x:c r="F97" s="4"/>
+      <x:c r="F97" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="46" customHeight="1">
       <x:c r="A98" s="4" t="str">
@@ -2761,7 +3187,9 @@
       <x:c r="E98" s="4" t="str">
         <x:v>https://github.com/bpg/terraform-provider-proxmox/compare/v0.94.0...v0.95.0</x:v>
       </x:c>
-      <x:c r="F98" s="4"/>
+      <x:c r="F98" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="46" customHeight="1">
       <x:c r="A99" s="4" t="str">
@@ -2779,7 +3207,9 @@
       <x:c r="E99" s="4" t="str">
         <x:v>https://github.com/bpg/terraform-provider-proxmox/compare/v0.97.1...v0.98.0</x:v>
       </x:c>
-      <x:c r="F99" s="4"/>
+      <x:c r="F99" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="46" customHeight="1">
       <x:c r="A100" s="4" t="str">
@@ -2797,7 +3227,9 @@
       <x:c r="E100" s="4" t="str">
         <x:v>https://github.com/bpg/terraform-provider-proxmox/compare/v0.107.0...v0.108.0</x:v>
       </x:c>
-      <x:c r="F100" s="4"/>
+      <x:c r="F100" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="46" customHeight="1">
       <x:c r="A101" s="4" t="str">
@@ -2815,7 +3247,9 @@
       <x:c r="E101" s="4" t="str">
         <x:v>https://github.com/bpg/terraform-provider-proxmox/compare/v0.112.0...v0.113.1</x:v>
       </x:c>
-      <x:c r="F101" s="4"/>
+      <x:c r="F101" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="46" customHeight="1">
       <x:c r="A102" s="4" t="str">
@@ -2833,7 +3267,9 @@
       <x:c r="E102" s="4" t="str">
         <x:v>https://github.com/bubbuild/bub/compare/0.1.1...0.2.0</x:v>
       </x:c>
-      <x:c r="F102" s="4"/>
+      <x:c r="F102" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" ht="46" customHeight="1">
       <x:c r="A103" s="4" t="str">
@@ -2851,7 +3287,9 @@
       <x:c r="E103" s="4" t="str">
         <x:v>https://github.com/bubbuild/bub/compare/0.2.0...0.2.1</x:v>
       </x:c>
-      <x:c r="F103" s="4"/>
+      <x:c r="F103" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="46" customHeight="1">
       <x:c r="A104" s="4" t="str">
@@ -2869,7 +3307,9 @@
       <x:c r="E104" s="4" t="str">
         <x:v>https://github.com/bubbuild/bub/compare/0.3.3...0.3.4</x:v>
       </x:c>
-      <x:c r="F104" s="4"/>
+      <x:c r="F104" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="46" customHeight="1">
       <x:c r="A105" s="4" t="str">
@@ -2887,7 +3327,9 @@
       <x:c r="E105" s="4" t="str">
         <x:v>https://github.com/bubbuild/bub/compare/0.4.0...0.4.1</x:v>
       </x:c>
-      <x:c r="F105" s="4"/>
+      <x:c r="F105" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="46" customHeight="1">
       <x:c r="A106" s="4" t="str">
@@ -2905,7 +3347,9 @@
       <x:c r="E106" s="4" t="str">
         <x:v>https://github.com/bubbuild/bub/compare/0.4.2...0.4.3</x:v>
       </x:c>
-      <x:c r="F106" s="4"/>
+      <x:c r="F106" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" ht="46" customHeight="1">
       <x:c r="A107" s="4" t="str">
@@ -2921,7 +3365,9 @@
         <x:v>https://github.com/caezium/burrow/releases/tag/v0.4.0</x:v>
       </x:c>
       <x:c r="E107" s="4"/>
-      <x:c r="F107" s="4"/>
+      <x:c r="F107" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="46" customHeight="1">
       <x:c r="A108" s="4" t="str">
@@ -2939,7 +3385,9 @@
       <x:c r="E108" s="4" t="str">
         <x:v>https://github.com/caezium/burrow/compare/v0.7.0...v0.7.1</x:v>
       </x:c>
-      <x:c r="F108" s="4"/>
+      <x:c r="F108" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="46" customHeight="1">
       <x:c r="A109" s="4" t="str">
@@ -2957,7 +3405,9 @@
       <x:c r="E109" s="4" t="str">
         <x:v>https://github.com/caezium/burrow/compare/v0.7.1...v0.7.2</x:v>
       </x:c>
-      <x:c r="F109" s="4"/>
+      <x:c r="F109" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="110" ht="46" customHeight="1">
       <x:c r="A110" s="4" t="str">
@@ -2975,7 +3425,9 @@
       <x:c r="E110" s="4" t="str">
         <x:v>https://github.com/caezium/burrow/compare/v0.8.2...v0.8.3</x:v>
       </x:c>
-      <x:c r="F110" s="4"/>
+      <x:c r="F110" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="46" customHeight="1">
       <x:c r="A111" s="4" t="str">
@@ -2993,7 +3445,9 @@
       <x:c r="E111" s="4" t="str">
         <x:v>https://github.com/caezium/burrow/compare/v0.10.5...v0.11.0</x:v>
       </x:c>
-      <x:c r="F111" s="4"/>
+      <x:c r="F111" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="112" ht="46" customHeight="1">
       <x:c r="A112" s="4" t="str">
@@ -3011,7 +3465,9 @@
       <x:c r="E112" s="4" t="str">
         <x:v>https://github.com/ckan/ckan/compare/ckan-2.11.3...ckan-2.10.9</x:v>
       </x:c>
-      <x:c r="F112" s="4"/>
+      <x:c r="F112" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="113" ht="46" customHeight="1">
       <x:c r="A113" s="4" t="str">
@@ -3029,7 +3485,9 @@
       <x:c r="E113" s="4" t="str">
         <x:v>https://github.com/ckan/ckan/compare/ckan-2.10.9...ckan-2.11.4</x:v>
       </x:c>
-      <x:c r="F113" s="4"/>
+      <x:c r="F113" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="46" customHeight="1">
       <x:c r="A114" s="4" t="str">
@@ -3047,7 +3505,9 @@
       <x:c r="E114" s="4" t="str">
         <x:v>https://github.com/ckan/ckan/compare/ckan-2.11.4...ckan-2.11.5</x:v>
       </x:c>
-      <x:c r="F114" s="4"/>
+      <x:c r="F114" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="46" customHeight="1">
       <x:c r="A115" s="4" t="str">
@@ -3065,7 +3525,9 @@
       <x:c r="E115" s="4" t="str">
         <x:v>https://github.com/ckan/ckan/compare/ckan-2.10.10...ckan-2.12.0</x:v>
       </x:c>
-      <x:c r="F115" s="4"/>
+      <x:c r="F115" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="46" customHeight="1">
       <x:c r="A116" s="4" t="str">
@@ -3083,7 +3545,9 @@
       <x:c r="E116" s="4" t="str">
         <x:v>https://github.com/ckan/ckan/compare/ckan-2.12.0...ckan-2.11.6</x:v>
       </x:c>
-      <x:c r="F116" s="4"/>
+      <x:c r="F116" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="46" customHeight="1">
       <x:c r="A117" s="4" t="str">
@@ -3101,7 +3565,9 @@
       <x:c r="E117" s="4" t="str">
         <x:v>https://github.com/copilot-emacs/copilot.el/compare/v0.2.0...v0.3.0</x:v>
       </x:c>
-      <x:c r="F117" s="4"/>
+      <x:c r="F117" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="46" customHeight="1">
       <x:c r="A118" s="4" t="str">
@@ -3119,7 +3585,9 @@
       <x:c r="E118" s="4" t="str">
         <x:v>https://github.com/copilot-emacs/copilot.el/compare/v0.3.0...v0.4.0</x:v>
       </x:c>
-      <x:c r="F118" s="4"/>
+      <x:c r="F118" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="119" ht="46" customHeight="1">
       <x:c r="A119" s="4" t="str">
@@ -3137,7 +3605,9 @@
       <x:c r="E119" s="4" t="str">
         <x:v>https://github.com/copilot-emacs/copilot.el/compare/v0.4.0...v0.5.0</x:v>
       </x:c>
-      <x:c r="F119" s="4"/>
+      <x:c r="F119" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="120" ht="46" customHeight="1">
       <x:c r="A120" s="4" t="str">
@@ -3155,7 +3625,9 @@
       <x:c r="E120" s="4" t="str">
         <x:v>https://github.com/copilot-emacs/copilot.el/compare/v0.6.0...v0.7.0</x:v>
       </x:c>
-      <x:c r="F120" s="4"/>
+      <x:c r="F120" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="121" ht="46" customHeight="1">
       <x:c r="A121" s="4" t="str">
@@ -3173,7 +3645,9 @@
       <x:c r="E121" s="4" t="str">
         <x:v>https://github.com/copilot-emacs/copilot.el/compare/v0.7.0...v0.8.0</x:v>
       </x:c>
-      <x:c r="F121" s="4"/>
+      <x:c r="F121" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="46" customHeight="1">
       <x:c r="A122" s="4" t="str">
@@ -3191,7 +3665,9 @@
       <x:c r="E122" s="4" t="str">
         <x:v>https://github.com/crate/crate/compare/5.10.15...6.0.4</x:v>
       </x:c>
-      <x:c r="F122" s="4"/>
+      <x:c r="F122" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="46" customHeight="1">
       <x:c r="A123" s="4" t="str">
@@ -3209,7 +3685,9 @@
       <x:c r="E123" s="4" t="str">
         <x:v>https://github.com/crate/crate/compare/6.2.3...6.2.4</x:v>
       </x:c>
-      <x:c r="F123" s="4"/>
+      <x:c r="F123" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="124" ht="46" customHeight="1">
       <x:c r="A124" s="4" t="str">
@@ -3227,7 +3705,9 @@
       <x:c r="E124" s="4" t="str">
         <x:v>https://github.com/crate/crate/compare/6.0.8...6.4.0</x:v>
       </x:c>
-      <x:c r="F124" s="4"/>
+      <x:c r="F124" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="46" customHeight="1">
       <x:c r="A125" s="4" t="str">
@@ -3245,7 +3725,9 @@
       <x:c r="E125" s="4" t="str">
         <x:v>https://github.com/crate/crate/compare/6.4.1...6.3.7</x:v>
       </x:c>
-      <x:c r="F125" s="4"/>
+      <x:c r="F125" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="46" customHeight="1">
       <x:c r="A126" s="4" t="str">
@@ -3263,7 +3745,9 @@
       <x:c r="E126" s="4" t="str">
         <x:v>https://github.com/crate/crate/compare/6.4.3...6.4.4</x:v>
       </x:c>
-      <x:c r="F126" s="4"/>
+      <x:c r="F126" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="46" customHeight="1">
       <x:c r="A127" s="4" t="str">
@@ -3281,7 +3765,9 @@
       <x:c r="E127" s="4" t="str">
         <x:v>https://github.com/cypress-io/github-action/compare/v6.10.2...v6.10.3</x:v>
       </x:c>
-      <x:c r="F127" s="4"/>
+      <x:c r="F127" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="46" customHeight="1">
       <x:c r="A128" s="4" t="str">
@@ -3299,7 +3785,9 @@
       <x:c r="E128" s="4" t="str">
         <x:v>https://github.com/cypress-io/github-action/compare/v7.0.0...v7.1.1</x:v>
       </x:c>
-      <x:c r="F128" s="4"/>
+      <x:c r="F128" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="129" ht="46" customHeight="1">
       <x:c r="A129" s="4" t="str">
@@ -3317,7 +3805,9 @@
       <x:c r="E129" s="4" t="str">
         <x:v>https://github.com/cypress-io/github-action/compare/v7.1.3...v7.1.4</x:v>
       </x:c>
-      <x:c r="F129" s="4"/>
+      <x:c r="F129" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="130" ht="46" customHeight="1">
       <x:c r="A130" s="4" t="str">
@@ -3335,7 +3825,9 @@
       <x:c r="E130" s="4" t="str">
         <x:v>https://github.com/cypress-io/github-action/compare/v7.1.8...v7.1.9</x:v>
       </x:c>
-      <x:c r="F130" s="4"/>
+      <x:c r="F130" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="131" ht="46" customHeight="1">
       <x:c r="A131" s="4" t="str">
@@ -3353,7 +3845,9 @@
       <x:c r="E131" s="4" t="str">
         <x:v>https://github.com/cypress-io/github-action/compare/v7.4.3...v7.4.4</x:v>
       </x:c>
-      <x:c r="F131" s="4"/>
+      <x:c r="F131" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="132" ht="46" customHeight="1">
       <x:c r="A132" s="4" t="str">
@@ -3371,7 +3865,9 @@
       <x:c r="E132" s="4" t="str">
         <x:v>https://github.com/deer-flow/llm-space/compare/v4.2.0...v4.2.1</x:v>
       </x:c>
-      <x:c r="F132" s="4"/>
+      <x:c r="F132" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="133" ht="46" customHeight="1">
       <x:c r="A133" s="4" t="str">
@@ -3389,7 +3885,9 @@
       <x:c r="E133" s="4" t="str">
         <x:v>https://github.com/deer-flow/llm-space/compare/v4.6.2...v4.6.3</x:v>
       </x:c>
-      <x:c r="F133" s="4"/>
+      <x:c r="F133" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="134" ht="46" customHeight="1">
       <x:c r="A134" s="4" t="str">
@@ -3407,7 +3905,9 @@
       <x:c r="E134" s="4" t="str">
         <x:v>https://github.com/deer-flow/llm-space/compare/v4.14.1...v4.14.2</x:v>
       </x:c>
-      <x:c r="F134" s="4"/>
+      <x:c r="F134" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="135" ht="46" customHeight="1">
       <x:c r="A135" s="4" t="str">
@@ -3425,7 +3925,9 @@
       <x:c r="E135" s="4" t="str">
         <x:v>https://github.com/deer-flow/llm-space/compare/v4.15.1...v4.15.2</x:v>
       </x:c>
-      <x:c r="F135" s="4"/>
+      <x:c r="F135" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="136" ht="46" customHeight="1">
       <x:c r="A136" s="4" t="str">
@@ -3443,7 +3945,9 @@
       <x:c r="E136" s="4" t="str">
         <x:v>https://github.com/deer-flow/llm-space/compare/v4.17.0...v4.18.0</x:v>
       </x:c>
-      <x:c r="F136" s="4"/>
+      <x:c r="F136" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="137" ht="46" customHeight="1">
       <x:c r="A137" s="4" t="str">
@@ -3461,7 +3965,9 @@
       <x:c r="E137" s="4" t="str">
         <x:v>https://github.com/googleads/googleads-mobile-ios-examples/compare/12.11.0...12.12.0</x:v>
       </x:c>
-      <x:c r="F137" s="4"/>
+      <x:c r="F137" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="138" ht="46" customHeight="1">
       <x:c r="A138" s="4" t="str">
@@ -3479,7 +3985,9 @@
       <x:c r="E138" s="4" t="str">
         <x:v>https://github.com/googleads/googleads-mobile-ios-examples/compare/13.1.0...13.2.0</x:v>
       </x:c>
-      <x:c r="F138" s="4"/>
+      <x:c r="F138" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="139" ht="46" customHeight="1">
       <x:c r="A139" s="4" t="str">
@@ -3497,7 +4005,9 @@
       <x:c r="E139" s="4" t="str">
         <x:v>https://github.com/googleads/googleads-mobile-ios-examples/compare/13.5.0...13.6.0</x:v>
       </x:c>
-      <x:c r="F139" s="4"/>
+      <x:c r="F139" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="140" ht="46" customHeight="1">
       <x:c r="A140" s="4" t="str">
@@ -3515,7 +4025,9 @@
       <x:c r="E140" s="4" t="str">
         <x:v>https://github.com/googleads/googleads-mobile-ios-examples/compare/13.7.0...13.8.0</x:v>
       </x:c>
-      <x:c r="F140" s="4"/>
+      <x:c r="F140" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="46" customHeight="1">
       <x:c r="A141" s="4" t="str">
@@ -3533,7 +4045,9 @@
       <x:c r="E141" s="4" t="str">
         <x:v>https://github.com/googleads/googleads-mobile-ios-examples/compare/13.8.0...13.9.0</x:v>
       </x:c>
-      <x:c r="F141" s="4"/>
+      <x:c r="F141" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="142" ht="46" customHeight="1">
       <x:c r="A142" s="4" t="str">
@@ -3549,7 +4063,9 @@
         <x:v>https://github.com/guhcostan/mac-cleaner-cli/releases/tag/v1.0.0</x:v>
       </x:c>
       <x:c r="E142" s="4"/>
-      <x:c r="F142" s="4"/>
+      <x:c r="F142" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="143" ht="46" customHeight="1">
       <x:c r="A143" s="4" t="str">
@@ -3567,7 +4083,9 @@
       <x:c r="E143" s="4" t="str">
         <x:v>https://github.com/guhcostan/mac-cleaner-cli/compare/v1.0.0...v1.1.0</x:v>
       </x:c>
-      <x:c r="F143" s="4"/>
+      <x:c r="F143" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="144" ht="46" customHeight="1">
       <x:c r="A144" s="4" t="str">
@@ -3585,7 +4103,9 @@
       <x:c r="E144" s="4" t="str">
         <x:v>https://github.com/guhcostan/mac-cleaner-cli/compare/v1.1.1...v1.1.2</x:v>
       </x:c>
-      <x:c r="F144" s="4"/>
+      <x:c r="F144" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="145" ht="46" customHeight="1">
       <x:c r="A145" s="4" t="str">
@@ -3603,7 +4123,9 @@
       <x:c r="E145" s="4" t="str">
         <x:v>https://github.com/guhcostan/mac-cleaner-cli/compare/v1.1.3...v1.1.4</x:v>
       </x:c>
-      <x:c r="F145" s="4"/>
+      <x:c r="F145" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="146" ht="46" customHeight="1">
       <x:c r="A146" s="4" t="str">
@@ -3621,7 +4143,9 @@
       <x:c r="E146" s="4" t="str">
         <x:v>https://github.com/guhcostan/mac-cleaner-cli/compare/v1.1.6...v1.1.7</x:v>
       </x:c>
-      <x:c r="F146" s="4"/>
+      <x:c r="F146" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="147" ht="46" customHeight="1">
       <x:c r="A147" s="4" t="str">
@@ -3637,7 +4161,9 @@
         <x:v>https://github.com/hardbeat920/monocode/releases/tag/v0.1.0</x:v>
       </x:c>
       <x:c r="E147" s="4"/>
-      <x:c r="F147" s="4"/>
+      <x:c r="F147" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="148" ht="46" customHeight="1">
       <x:c r="A148" s="4" t="str">
@@ -3655,7 +4181,9 @@
       <x:c r="E148" s="4" t="str">
         <x:v>https://github.com/hardbeat920/monocode/compare/v0.1.4...v0.1.5</x:v>
       </x:c>
-      <x:c r="F148" s="4"/>
+      <x:c r="F148" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="149" ht="46" customHeight="1">
       <x:c r="A149" s="4" t="str">
@@ -3673,7 +4201,9 @@
       <x:c r="E149" s="4" t="str">
         <x:v>https://github.com/hardbeat920/monocode/compare/v0.1.43...v0.1.44</x:v>
       </x:c>
-      <x:c r="F149" s="4"/>
+      <x:c r="F149" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="150" ht="46" customHeight="1">
       <x:c r="A150" s="4" t="str">
@@ -3691,7 +4221,9 @@
       <x:c r="E150" s="4" t="str">
         <x:v>https://github.com/hardbeat920/monocode/compare/v0.1.51...v0.1.52</x:v>
       </x:c>
-      <x:c r="F150" s="4"/>
+      <x:c r="F150" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="151" ht="46" customHeight="1">
       <x:c r="A151" s="4" t="str">
@@ -3709,7 +4241,9 @@
       <x:c r="E151" s="4" t="str">
         <x:v>https://github.com/hardbeat920/monocode/compare/v0.2.0...v0.3.0</x:v>
       </x:c>
-      <x:c r="F151" s="4"/>
+      <x:c r="F151" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="46" customHeight="1">
       <x:c r="A152" s="4" t="str">
@@ -3727,7 +4261,9 @@
       <x:c r="E152" s="4" t="str">
         <x:v>https://github.com/htmlhint/HTMLHint/compare/v1.7.1...v1.8.0</x:v>
       </x:c>
-      <x:c r="F152" s="4"/>
+      <x:c r="F152" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="46" customHeight="1">
       <x:c r="A153" s="4" t="str">
@@ -3745,7 +4281,9 @@
       <x:c r="E153" s="4" t="str">
         <x:v>https://github.com/htmlhint/HTMLHint/compare/v1.8.0...v1.8.1</x:v>
       </x:c>
-      <x:c r="F153" s="4"/>
+      <x:c r="F153" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="154" ht="46" customHeight="1">
       <x:c r="A154" s="4" t="str">
@@ -3763,7 +4301,9 @@
       <x:c r="E154" s="4" t="str">
         <x:v>https://github.com/htmlhint/HTMLHint/compare/v1.8.1...v1.9.0</x:v>
       </x:c>
-      <x:c r="F154" s="4"/>
+      <x:c r="F154" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="155" ht="46" customHeight="1">
       <x:c r="A155" s="4" t="str">
@@ -3781,7 +4321,9 @@
       <x:c r="E155" s="4" t="str">
         <x:v>https://github.com/htmlhint/HTMLHint/compare/v1.9.0...v1.9.1</x:v>
       </x:c>
-      <x:c r="F155" s="4"/>
+      <x:c r="F155" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="156" ht="46" customHeight="1">
       <x:c r="A156" s="4" t="str">
@@ -3799,7 +4341,9 @@
       <x:c r="E156" s="4" t="str">
         <x:v>https://github.com/htmlhint/HTMLHint/compare/v1.9.1...v1.9.2</x:v>
       </x:c>
-      <x:c r="F156" s="4"/>
+      <x:c r="F156" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="157" ht="46" customHeight="1">
       <x:c r="A157" s="4" t="str">
@@ -3817,7 +4361,9 @@
       <x:c r="E157" s="4" t="str">
         <x:v>https://github.com/jenkinsci/docker/compare/2.530...2.531</x:v>
       </x:c>
-      <x:c r="F157" s="4"/>
+      <x:c r="F157" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="158" ht="46" customHeight="1">
       <x:c r="A158" s="4" t="str">
@@ -3835,7 +4381,9 @@
       <x:c r="E158" s="4" t="str">
         <x:v>https://github.com/jenkinsci/docker/compare/2.534...2.535</x:v>
       </x:c>
-      <x:c r="F158" s="4"/>
+      <x:c r="F158" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="159" ht="46" customHeight="1">
       <x:c r="A159" s="4" t="str">
@@ -3853,7 +4401,9 @@
       <x:c r="E159" s="4" t="str">
         <x:v>https://github.com/jenkinsci/docker/compare/2.567...2.568</x:v>
       </x:c>
-      <x:c r="F159" s="4"/>
+      <x:c r="F159" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="160" ht="46" customHeight="1">
       <x:c r="A160" s="4" t="str">
@@ -3871,7 +4421,9 @@
       <x:c r="E160" s="4" t="str">
         <x:v>https://github.com/jenkinsci/docker/compare/2.574...2.575</x:v>
       </x:c>
-      <x:c r="F160" s="4"/>
+      <x:c r="F160" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="161" ht="46" customHeight="1">
       <x:c r="A161" s="4" t="str">
@@ -3889,7 +4441,9 @@
       <x:c r="E161" s="4" t="str">
         <x:v>https://github.com/jenkinsci/docker/compare/2.581...2.582</x:v>
       </x:c>
-      <x:c r="F161" s="4"/>
+      <x:c r="F161" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="46" customHeight="1">
       <x:c r="A162" s="4" t="str">
@@ -3907,7 +4461,9 @@
       <x:c r="E162" s="4" t="str">
         <x:v>https://github.com/jhomlala/betterplayer/compare/1.0.0...1.0.1</x:v>
       </x:c>
-      <x:c r="F162" s="4"/>
+      <x:c r="F162" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="163" ht="46" customHeight="1">
       <x:c r="A163" s="4" t="str">
@@ -3925,7 +4481,9 @@
       <x:c r="E163" s="4" t="str">
         <x:v>https://github.com/jhomlala/betterplayer/compare/1.1.0...1.1.1</x:v>
       </x:c>
-      <x:c r="F163" s="4"/>
+      <x:c r="F163" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="164" ht="46" customHeight="1">
       <x:c r="A164" s="4" t="str">
@@ -3943,7 +4501,9 @@
       <x:c r="E164" s="4" t="str">
         <x:v>https://github.com/jhomlala/betterplayer/compare/1.5.1...1.6.0</x:v>
       </x:c>
-      <x:c r="F164" s="4"/>
+      <x:c r="F164" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="165" ht="46" customHeight="1">
       <x:c r="A165" s="4" t="str">
@@ -3961,7 +4521,9 @@
       <x:c r="E165" s="4" t="str">
         <x:v>https://github.com/jhomlala/betterplayer/compare/1.8.0...1.8.1</x:v>
       </x:c>
-      <x:c r="F165" s="4"/>
+      <x:c r="F165" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="166" ht="46" customHeight="1">
       <x:c r="A166" s="4" t="str">
@@ -3979,7 +4541,9 @@
       <x:c r="E166" s="4" t="str">
         <x:v>https://github.com/jhomlala/betterplayer/compare/1.9.0...1.10.0</x:v>
       </x:c>
-      <x:c r="F166" s="4"/>
+      <x:c r="F166" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="167" ht="46" customHeight="1">
       <x:c r="A167" s="4" t="str">
@@ -3997,7 +4561,9 @@
       <x:c r="E167" s="4" t="str">
         <x:v>https://github.com/kubeshop/testkube/compare/2.4.2...2.4.3</x:v>
       </x:c>
-      <x:c r="F167" s="4"/>
+      <x:c r="F167" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="168" ht="46" customHeight="1">
       <x:c r="A168" s="4" t="str">
@@ -4015,7 +4581,9 @@
       <x:c r="E168" s="4" t="str">
         <x:v>https://github.com/kubeshop/testkube/compare/2.5.1...2.5.2</x:v>
       </x:c>
-      <x:c r="F168" s="4"/>
+      <x:c r="F168" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="169" ht="46" customHeight="1">
       <x:c r="A169" s="4" t="str">
@@ -4033,7 +4601,9 @@
       <x:c r="E169" s="4" t="str">
         <x:v>https://github.com/kubeshop/testkube/compare/2.5.6...2.5.7</x:v>
       </x:c>
-      <x:c r="F169" s="4"/>
+      <x:c r="F169" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="170" ht="46" customHeight="1">
       <x:c r="A170" s="4" t="str">
@@ -4051,7 +4621,9 @@
       <x:c r="E170" s="4" t="str">
         <x:v>https://github.com/kubeshop/testkube/compare/2.8.3...2.9.0</x:v>
       </x:c>
-      <x:c r="F170" s="4"/>
+      <x:c r="F170" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="171" ht="46" customHeight="1">
       <x:c r="A171" s="4" t="str">
@@ -4069,7 +4641,9 @@
       <x:c r="E171" s="4" t="str">
         <x:v>https://github.com/kubeshop/testkube/compare/2.9.0...2.9.1</x:v>
       </x:c>
-      <x:c r="F171" s="4"/>
+      <x:c r="F171" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="172" ht="46" customHeight="1">
       <x:c r="A172" s="4" t="str">
@@ -4087,7 +4661,9 @@
       <x:c r="E172" s="4" t="str">
         <x:v>https://github.com/liveblocks/liveblocks/compare/v3.15.5...v3.16.0</x:v>
       </x:c>
-      <x:c r="F172" s="4"/>
+      <x:c r="F172" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="173" ht="46" customHeight="1">
       <x:c r="A173" s="4" t="str">
@@ -4105,7 +4681,9 @@
       <x:c r="E173" s="4" t="str">
         <x:v>https://github.com/liveblocks/liveblocks/compare/v3.17.0...v3.18.0</x:v>
       </x:c>
-      <x:c r="F173" s="4"/>
+      <x:c r="F173" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="174" ht="46" customHeight="1">
       <x:c r="A174" s="4" t="str">
@@ -4123,7 +4701,9 @@
       <x:c r="E174" s="4" t="str">
         <x:v>https://github.com/liveblocks/liveblocks/compare/v3.18.0...v3.18.1</x:v>
       </x:c>
-      <x:c r="F174" s="4"/>
+      <x:c r="F174" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="175" ht="46" customHeight="1">
       <x:c r="A175" s="4" t="str">
@@ -4141,7 +4721,9 @@
       <x:c r="E175" s="4" t="str">
         <x:v>https://github.com/liveblocks/liveblocks/compare/v3.20.0...v3.20.1</x:v>
       </x:c>
-      <x:c r="F175" s="4"/>
+      <x:c r="F175" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="176" ht="46" customHeight="1">
       <x:c r="A176" s="4" t="str">
@@ -4159,7 +4741,9 @@
       <x:c r="E176" s="4" t="str">
         <x:v>https://github.com/liveblocks/liveblocks/compare/v3.23.0...v3.23.1</x:v>
       </x:c>
-      <x:c r="F176" s="4"/>
+      <x:c r="F176" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="177" ht="46" customHeight="1">
       <x:c r="A177" s="4" t="str">
@@ -4177,7 +4761,9 @@
       <x:c r="E177" s="4" t="str">
         <x:v>https://github.com/loro-dev/loro/compare/loro-crdt%401.8.1...loro-crdt%401.8.2</x:v>
       </x:c>
-      <x:c r="F177" s="4"/>
+      <x:c r="F177" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="178" ht="46" customHeight="1">
       <x:c r="A178" s="4" t="str">
@@ -4195,7 +4781,9 @@
       <x:c r="E178" s="4" t="str">
         <x:v>https://github.com/loro-dev/loro/compare/loro-crdt-map%401.10.3...loro-crdt%401.10.3</x:v>
       </x:c>
-      <x:c r="F178" s="4"/>
+      <x:c r="F178" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="179" ht="46" customHeight="1">
       <x:c r="A179" s="4" t="str">
@@ -4213,7 +4801,9 @@
       <x:c r="E179" s="4" t="str">
         <x:v>https://github.com/loro-dev/loro/compare/loro-crdt-map%401.10.5...loro-crdt%401.10.5</x:v>
       </x:c>
-      <x:c r="F179" s="4"/>
+      <x:c r="F179" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="180" ht="46" customHeight="1">
       <x:c r="A180" s="4" t="str">
@@ -4231,7 +4821,9 @@
       <x:c r="E180" s="4" t="str">
         <x:v>https://github.com/loro-dev/loro/compare/loro-crdt%401.11.0...loro-crdt-map%401.11.0</x:v>
       </x:c>
-      <x:c r="F180" s="4"/>
+      <x:c r="F180" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="181" ht="46" customHeight="1">
       <x:c r="A181" s="4" t="str">
@@ -4249,7 +4841,9 @@
       <x:c r="E181" s="4" t="str">
         <x:v>https://github.com/loro-dev/loro/compare/loro-crdt-map%401.11.0...loro-crdt-map%401.11.1</x:v>
       </x:c>
-      <x:c r="F181" s="4"/>
+      <x:c r="F181" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="182" ht="46" customHeight="1">
       <x:c r="A182" s="4" t="str">
@@ -4267,7 +4861,9 @@
       <x:c r="E182" s="4" t="str">
         <x:v>https://github.com/microsoft/mcp/compare/Template.Mcp.Server-0.0.12-alpha.6119543...Template.Mcp.Server-0.0.12-alpha.6120437</x:v>
       </x:c>
-      <x:c r="F182" s="4"/>
+      <x:c r="F182" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="183" ht="46" customHeight="1">
       <x:c r="A183" s="4" t="str">
@@ -4285,7 +4881,9 @@
       <x:c r="E183" s="4" t="str">
         <x:v>https://github.com/microsoft/mcp/compare/Template.Mcp.Server-0.0.12-alpha.6235263...Template.Mcp.Server-0.0.12-alpha.6223865</x:v>
       </x:c>
-      <x:c r="F183" s="4"/>
+      <x:c r="F183" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="184" ht="46" customHeight="1">
       <x:c r="A184" s="4" t="str">
@@ -4303,7 +4901,9 @@
       <x:c r="E184" s="4" t="str">
         <x:v>https://github.com/microsoft/mcp/compare/Fabric.Mcp.Server-1.3.0...Azure.Mcp.Server-3.0.0-beta.34</x:v>
       </x:c>
-      <x:c r="F184" s="4"/>
+      <x:c r="F184" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="185" ht="46" customHeight="1">
       <x:c r="A185" s="4" t="str">
@@ -4321,7 +4921,9 @@
       <x:c r="E185" s="4" t="str">
         <x:v>https://github.com/microsoft/mcp/compare/Azure.Mcp.Server-3.0.0-beta.37...Azure.Mcp.Server-3.0.0-beta.38</x:v>
       </x:c>
-      <x:c r="F185" s="4"/>
+      <x:c r="F185" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="186" ht="46" customHeight="1">
       <x:c r="A186" s="4" t="str">
@@ -4339,7 +4941,9 @@
       <x:c r="E186" s="4" t="str">
         <x:v>https://github.com/microsoft/mcp/compare/Azure.Mcp.Server-3.0.0-beta.38...Fabric.Mcp.Server-1.4.0</x:v>
       </x:c>
-      <x:c r="F186" s="4"/>
+      <x:c r="F186" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="187" ht="46" customHeight="1">
       <x:c r="A187" s="4" t="str">
@@ -4357,7 +4961,9 @@
       <x:c r="E187" s="4" t="str">
         <x:v>https://github.com/mivano/azure-cost-cli/compare/0.50.0...0.51.0</x:v>
       </x:c>
-      <x:c r="F187" s="4"/>
+      <x:c r="F187" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="188" ht="46" customHeight="1">
       <x:c r="A188" s="4" t="str">
@@ -4375,7 +4981,9 @@
       <x:c r="E188" s="4" t="str">
         <x:v>https://github.com/mivano/azure-cost-cli/compare/0.51.0...0.52.0</x:v>
       </x:c>
-      <x:c r="F188" s="4"/>
+      <x:c r="F188" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="189" ht="46" customHeight="1">
       <x:c r="A189" s="4" t="str">
@@ -4393,7 +5001,9 @@
       <x:c r="E189" s="4" t="str">
         <x:v>https://github.com/mivano/azure-cost-cli/compare/0.55.0...0.56.0</x:v>
       </x:c>
-      <x:c r="F189" s="4"/>
+      <x:c r="F189" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="190" ht="46" customHeight="1">
       <x:c r="A190" s="4" t="str">
@@ -4411,7 +5021,9 @@
       <x:c r="E190" s="4" t="str">
         <x:v>https://github.com/mivano/azure-cost-cli/compare/0.57.0...0.58.0</x:v>
       </x:c>
-      <x:c r="F190" s="4"/>
+      <x:c r="F190" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="191" ht="46" customHeight="1">
       <x:c r="A191" s="4" t="str">
@@ -4429,7 +5041,9 @@
       <x:c r="E191" s="4" t="str">
         <x:v>https://github.com/mivano/azure-cost-cli/compare/0.58.0...0.59.0</x:v>
       </x:c>
-      <x:c r="F191" s="4"/>
+      <x:c r="F191" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="192" ht="46" customHeight="1">
       <x:c r="A192" s="4" t="str">
@@ -4447,7 +5061,9 @@
       <x:c r="E192" s="4" t="str">
         <x:v>https://github.com/mozilla/pontoon/compare/2018-12-19...v2026.08.19</x:v>
       </x:c>
-      <x:c r="F192" s="4"/>
+      <x:c r="F192" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="193" ht="46" customHeight="1">
       <x:c r="A193" s="4" t="str">
@@ -4465,7 +5081,9 @@
       <x:c r="E193" s="4" t="str">
         <x:v>https://github.com/mozilla/pontoon/compare/v2026.08.19...v2026.08.25</x:v>
       </x:c>
-      <x:c r="F193" s="4"/>
+      <x:c r="F193" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="194" ht="46" customHeight="1">
       <x:c r="A194" s="4" t="str">
@@ -4483,7 +5101,9 @@
       <x:c r="E194" s="4" t="str">
         <x:v>https://github.com/mozilla/pontoon/compare/v2026.08.31...v2026.09.02</x:v>
       </x:c>
-      <x:c r="F194" s="4"/>
+      <x:c r="F194" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="195" ht="46" customHeight="1">
       <x:c r="A195" s="4" t="str">
@@ -4501,7 +5121,9 @@
       <x:c r="E195" s="4" t="str">
         <x:v>https://github.com/mozilla/pontoon/compare/v2026.09.14...v2026.09.15</x:v>
       </x:c>
-      <x:c r="F195" s="4"/>
+      <x:c r="F195" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="196" ht="46" customHeight="1">
       <x:c r="A196" s="4" t="str">
@@ -4519,7 +5141,9 @@
       <x:c r="E196" s="4" t="str">
         <x:v>https://github.com/mozilla/pontoon/compare/v2026.09.21...v2026.09.22</x:v>
       </x:c>
-      <x:c r="F196" s="4"/>
+      <x:c r="F196" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="197" ht="46" customHeight="1">
       <x:c r="A197" s="4" t="str">
@@ -4537,7 +5161,9 @@
       <x:c r="E197" s="4" t="str">
         <x:v>https://github.com/node-opcua/node-opcua/compare/v2.157.0...v2.158.0</x:v>
       </x:c>
-      <x:c r="F197" s="4"/>
+      <x:c r="F197" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="198" ht="46" customHeight="1">
       <x:c r="A198" s="4" t="str">
@@ -4555,7 +5181,9 @@
       <x:c r="E198" s="4" t="str">
         <x:v>https://github.com/node-opcua/node-opcua/compare/v2.165.1...v2.167.0</x:v>
       </x:c>
-      <x:c r="F198" s="4"/>
+      <x:c r="F198" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="199" ht="46" customHeight="1">
       <x:c r="A199" s="4" t="str">
@@ -4573,7 +5201,9 @@
       <x:c r="E199" s="4" t="str">
         <x:v>https://github.com/node-opcua/node-opcua/compare/v2.167.0...v2.168.0</x:v>
       </x:c>
-      <x:c r="F199" s="4"/>
+      <x:c r="F199" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="200" ht="46" customHeight="1">
       <x:c r="A200" s="4" t="str">
@@ -4591,7 +5221,9 @@
       <x:c r="E200" s="4" t="str">
         <x:v>https://github.com/node-opcua/node-opcua/compare/v2.179.0...v2.180.0</x:v>
       </x:c>
-      <x:c r="F200" s="4"/>
+      <x:c r="F200" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="201" ht="46" customHeight="1">
       <x:c r="A201" s="4" t="str">
@@ -4609,7 +5241,9 @@
       <x:c r="E201" s="4" t="str">
         <x:v>https://github.com/node-opcua/node-opcua/compare/v2.183.0...v2.184.0</x:v>
       </x:c>
-      <x:c r="F201" s="4"/>
+      <x:c r="F201" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="202" ht="46" customHeight="1">
       <x:c r="A202" s="4" t="str">
@@ -4627,7 +5261,9 @@
       <x:c r="E202" s="4" t="str">
         <x:v>https://github.com/odygrd/quill/compare/v10.1.0...v10.2.0</x:v>
       </x:c>
-      <x:c r="F202" s="4"/>
+      <x:c r="F202" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="203" ht="46" customHeight="1">
       <x:c r="A203" s="4" t="str">
@@ -4645,7 +5281,9 @@
       <x:c r="E203" s="4" t="str">
         <x:v>https://github.com/odygrd/quill/compare/v11.0.0...v11.0.1</x:v>
       </x:c>
-      <x:c r="F203" s="4"/>
+      <x:c r="F203" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="204" ht="46" customHeight="1">
       <x:c r="A204" s="4" t="str">
@@ -4663,7 +5301,9 @@
       <x:c r="E204" s="4" t="str">
         <x:v>https://github.com/odygrd/quill/compare/v11.1.0...v12.0.0</x:v>
       </x:c>
-      <x:c r="F204" s="4"/>
+      <x:c r="F204" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="205" ht="46" customHeight="1">
       <x:c r="A205" s="4" t="str">
@@ -4681,7 +5321,9 @@
       <x:c r="E205" s="4" t="str">
         <x:v>https://github.com/odygrd/quill/compare/v12.2.1...v12.2.2</x:v>
       </x:c>
-      <x:c r="F205" s="4"/>
+      <x:c r="F205" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="206" ht="46" customHeight="1">
       <x:c r="A206" s="4" t="str">
@@ -4699,7 +5341,9 @@
       <x:c r="E206" s="4" t="str">
         <x:v>https://github.com/odygrd/quill/compare/v12.2.2...v13.0.0</x:v>
       </x:c>
-      <x:c r="F206" s="4"/>
+      <x:c r="F206" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="207" ht="46" customHeight="1">
       <x:c r="A207" s="4" t="str">
@@ -4717,7 +5361,9 @@
       <x:c r="E207" s="4" t="str">
         <x:v>https://github.com/open-logic/open-logic/compare/4.1.0...4.2.0</x:v>
       </x:c>
-      <x:c r="F207" s="4"/>
+      <x:c r="F207" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="208" ht="46" customHeight="1">
       <x:c r="A208" s="4" t="str">
@@ -4735,7 +5381,9 @@
       <x:c r="E208" s="4" t="str">
         <x:v>https://github.com/open-logic/open-logic/compare/4.2.0...4.3.0</x:v>
       </x:c>
-      <x:c r="F208" s="4"/>
+      <x:c r="F208" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="209" ht="46" customHeight="1">
       <x:c r="A209" s="4" t="str">
@@ -4753,7 +5401,9 @@
       <x:c r="E209" s="4" t="str">
         <x:v>https://github.com/open-logic/open-logic/compare/4.3.0...4.4.0</x:v>
       </x:c>
-      <x:c r="F209" s="4"/>
+      <x:c r="F209" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="210" ht="46" customHeight="1">
       <x:c r="A210" s="4" t="str">
@@ -4771,7 +5421,9 @@
       <x:c r="E210" s="4" t="str">
         <x:v>https://github.com/open-logic/open-logic/compare/4.4.1...4.5.0</x:v>
       </x:c>
-      <x:c r="F210" s="4"/>
+      <x:c r="F210" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="211" ht="46" customHeight="1">
       <x:c r="A211" s="4" t="str">
@@ -4789,7 +5441,9 @@
       <x:c r="E211" s="4" t="str">
         <x:v>https://github.com/open-logic/open-logic/compare/4.5.0...4.6.0</x:v>
       </x:c>
-      <x:c r="F211" s="4"/>
+      <x:c r="F211" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="212" ht="46" customHeight="1">
       <x:c r="A212" s="4" t="str">
@@ -4807,7 +5461,9 @@
       <x:c r="E212" s="4" t="str">
         <x:v>https://github.com/opengeos/geoai/compare/v0.32.0...v0.33.0</x:v>
       </x:c>
-      <x:c r="F212" s="4"/>
+      <x:c r="F212" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="213" ht="46" customHeight="1">
       <x:c r="A213" s="4" t="str">
@@ -4825,7 +5481,9 @@
       <x:c r="E213" s="4" t="str">
         <x:v>https://github.com/opengeos/geoai/compare/v0.33.0...v0.34.0</x:v>
       </x:c>
-      <x:c r="F213" s="4"/>
+      <x:c r="F213" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="214" ht="46" customHeight="1">
       <x:c r="A214" s="4" t="str">
@@ -4843,7 +5501,9 @@
       <x:c r="E214" s="4" t="str">
         <x:v>https://github.com/opengeos/geoai/compare/v0.39.1...v0.39.2</x:v>
       </x:c>
-      <x:c r="F214" s="4"/>
+      <x:c r="F214" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="215" ht="46" customHeight="1">
       <x:c r="A215" s="4" t="str">
@@ -4861,7 +5521,9 @@
       <x:c r="E215" s="4" t="str">
         <x:v>https://github.com/opengeos/geoai/compare/v0.40.0...v0.40.1</x:v>
       </x:c>
-      <x:c r="F215" s="4"/>
+      <x:c r="F215" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="216" ht="46" customHeight="1">
       <x:c r="A216" s="4" t="str">
@@ -4879,7 +5541,9 @@
       <x:c r="E216" s="4" t="str">
         <x:v>https://github.com/opengeos/geoai/compare/v0.42.0...v0.43.0</x:v>
       </x:c>
-      <x:c r="F216" s="4"/>
+      <x:c r="F216" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="217" ht="46" customHeight="1">
       <x:c r="A217" s="4" t="str">
@@ -4897,7 +5561,9 @@
       <x:c r="E217" s="4" t="str">
         <x:v>https://github.com/pgjdbc/pgjdbc/compare/REL42.7.8...REL42.7.9</x:v>
       </x:c>
-      <x:c r="F217" s="4"/>
+      <x:c r="F217" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="218" ht="46" customHeight="1">
       <x:c r="A218" s="4" t="str">
@@ -4915,7 +5581,9 @@
       <x:c r="E218" s="4" t="str">
         <x:v>https://github.com/pgjdbc/pgjdbc/compare/REL42.7.9...REL42.7.10</x:v>
       </x:c>
-      <x:c r="F218" s="4"/>
+      <x:c r="F218" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="219" ht="46" customHeight="1">
       <x:c r="A219" s="4" t="str">
@@ -4933,7 +5601,9 @@
       <x:c r="E219" s="4" t="str">
         <x:v>https://github.com/pgjdbc/pgjdbc/compare/REL42.7.10...REL42.7.11</x:v>
       </x:c>
-      <x:c r="F219" s="4"/>
+      <x:c r="F219" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="220" ht="46" customHeight="1">
       <x:c r="A220" s="4" t="str">
@@ -4951,7 +5621,9 @@
       <x:c r="E220" s="4" t="str">
         <x:v>https://github.com/pgjdbc/pgjdbc/compare/REL42.7.11...REL42.7.12</x:v>
       </x:c>
-      <x:c r="F220" s="4"/>
+      <x:c r="F220" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="221" ht="46" customHeight="1">
       <x:c r="A221" s="4" t="str">
@@ -4969,7 +5641,9 @@
       <x:c r="E221" s="4" t="str">
         <x:v>https://github.com/pgjdbc/pgjdbc/compare/REL42.7.12...REL42.7.13</x:v>
       </x:c>
-      <x:c r="F221" s="4"/>
+      <x:c r="F221" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="222" ht="46" customHeight="1">
       <x:c r="A222" s="4" t="str">
@@ -4987,7 +5661,9 @@
       <x:c r="E222" s="4" t="str">
         <x:v>https://github.com/prebid/Prebid.js/compare/10.11.0...10.12.0</x:v>
       </x:c>
-      <x:c r="F222" s="4"/>
+      <x:c r="F222" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="223" ht="46" customHeight="1">
       <x:c r="A223" s="4" t="str">
@@ -5005,7 +5681,9 @@
       <x:c r="E223" s="4" t="str">
         <x:v>https://github.com/prebid/Prebid.js/compare/9.53.3...10.17.0</x:v>
       </x:c>
-      <x:c r="F223" s="4"/>
+      <x:c r="F223" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="224" ht="46" customHeight="1">
       <x:c r="A224" s="4" t="str">
@@ -5023,7 +5701,9 @@
       <x:c r="E224" s="4" t="str">
         <x:v>https://github.com/prebid/Prebid.js/compare/10.21.0...10.22.0</x:v>
       </x:c>
-      <x:c r="F224" s="4"/>
+      <x:c r="F224" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="225" ht="46" customHeight="1">
       <x:c r="A225" s="4" t="str">
@@ -5041,7 +5721,9 @@
       <x:c r="E225" s="4" t="str">
         <x:v>https://github.com/prebid/Prebid.js/compare/11.9.0...11.10.0</x:v>
       </x:c>
-      <x:c r="F225" s="4"/>
+      <x:c r="F225" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="226" ht="46" customHeight="1">
       <x:c r="A226" s="4" t="str">
@@ -5059,7 +5741,9 @@
       <x:c r="E226" s="4" t="str">
         <x:v>https://github.com/prebid/Prebid.js/compare/11.23.0...11.24.0</x:v>
       </x:c>
-      <x:c r="F226" s="4"/>
+      <x:c r="F226" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="227" ht="46" customHeight="1">
       <x:c r="A227" s="4" t="str">
@@ -5077,7 +5761,9 @@
       <x:c r="E227" s="4" t="str">
         <x:v>https://github.com/project-zot/zot/compare/v2.1.8...v2.1.9</x:v>
       </x:c>
-      <x:c r="F227" s="4"/>
+      <x:c r="F227" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="228" ht="46" customHeight="1">
       <x:c r="A228" s="4" t="str">
@@ -5095,7 +5781,9 @@
       <x:c r="E228" s="4" t="str">
         <x:v>https://github.com/project-zot/zot/compare/v2.1.13...v2.1.14</x:v>
       </x:c>
-      <x:c r="F228" s="4"/>
+      <x:c r="F228" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="229" ht="46" customHeight="1">
       <x:c r="A229" s="4" t="str">
@@ -5113,7 +5801,9 @@
       <x:c r="E229" s="4" t="str">
         <x:v>https://github.com/project-zot/zot/compare/v2.1.16...v2.1.17</x:v>
       </x:c>
-      <x:c r="F229" s="4"/>
+      <x:c r="F229" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="230" ht="46" customHeight="1">
       <x:c r="A230" s="4" t="str">
@@ -5131,7 +5821,9 @@
       <x:c r="E230" s="4" t="str">
         <x:v>https://github.com/project-zot/zot/compare/v2.1.17...v2.1.18</x:v>
       </x:c>
-      <x:c r="F230" s="4"/>
+      <x:c r="F230" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="231" ht="46" customHeight="1">
       <x:c r="A231" s="4" t="str">
@@ -5149,7 +5841,9 @@
       <x:c r="E231" s="4" t="str">
         <x:v>https://github.com/project-zot/zot/compare/v2.1.19...v2.1.20</x:v>
       </x:c>
-      <x:c r="F231" s="4"/>
+      <x:c r="F231" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="232" ht="46" customHeight="1">
       <x:c r="A232" s="4" t="str">
@@ -5165,7 +5859,9 @@
         <x:v>https://github.com/puemos/craftplan/releases/tag/v0.2.0</x:v>
       </x:c>
       <x:c r="E232" s="4"/>
-      <x:c r="F232" s="4"/>
+      <x:c r="F232" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="233" ht="46" customHeight="1">
       <x:c r="A233" s="4" t="str">
@@ -5183,7 +5879,9 @@
       <x:c r="E233" s="4" t="str">
         <x:v>https://github.com/puemos/craftplan/compare/v0.3.5...v0.3.6</x:v>
       </x:c>
-      <x:c r="F233" s="4"/>
+      <x:c r="F233" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="234" ht="46" customHeight="1">
       <x:c r="A234" s="4" t="str">
@@ -5201,7 +5899,9 @@
       <x:c r="E234" s="4" t="str">
         <x:v>https://github.com/puemos/craftplan/compare/v0.3.6...v0.3.7</x:v>
       </x:c>
-      <x:c r="F234" s="4"/>
+      <x:c r="F234" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="235" ht="46" customHeight="1">
       <x:c r="A235" s="4" t="str">
@@ -5219,7 +5919,9 @@
       <x:c r="E235" s="4" t="str">
         <x:v>https://github.com/puemos/craftplan/compare/v0.6.0...v0.6.1</x:v>
       </x:c>
-      <x:c r="F235" s="4"/>
+      <x:c r="F235" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="236" ht="46" customHeight="1">
       <x:c r="A236" s="4" t="str">
@@ -5237,7 +5939,9 @@
       <x:c r="E236" s="4" t="str">
         <x:v>https://github.com/puemos/craftplan/compare/v0.6.2...v0.6.3</x:v>
       </x:c>
-      <x:c r="F236" s="4"/>
+      <x:c r="F236" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="237" ht="46" customHeight="1">
       <x:c r="A237" s="4" t="str">
@@ -5255,7 +5959,9 @@
       <x:c r="E237" s="4" t="str">
         <x:v>https://github.com/puma/puma/compare/v7.0.3...v7.0.4</x:v>
       </x:c>
-      <x:c r="F237" s="4"/>
+      <x:c r="F237" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="238" ht="46" customHeight="1">
       <x:c r="A238" s="4" t="str">
@@ -5273,7 +5979,9 @@
       <x:c r="E238" s="4" t="str">
         <x:v>https://github.com/puma/puma/compare/v7.0.4...v7.1.0</x:v>
       </x:c>
-      <x:c r="F238" s="4"/>
+      <x:c r="F238" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="239" ht="46" customHeight="1">
       <x:c r="A239" s="4" t="str">
@@ -5291,7 +5999,9 @@
       <x:c r="E239" s="4" t="str">
         <x:v>https://github.com/puma/puma/compare/v7.1.0...v7.2.0</x:v>
       </x:c>
-      <x:c r="F239" s="4"/>
+      <x:c r="F239" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="240" ht="46" customHeight="1">
       <x:c r="A240" s="4" t="str">
@@ -5309,7 +6019,9 @@
       <x:c r="E240" s="4" t="str">
         <x:v>https://github.com/puma/puma/compare/v8.0.0...v8.0.1</x:v>
       </x:c>
-      <x:c r="F240" s="4"/>
+      <x:c r="F240" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="241" ht="46" customHeight="1">
       <x:c r="A241" s="4" t="str">
@@ -5327,7 +6039,9 @@
       <x:c r="E241" s="4" t="str">
         <x:v>https://github.com/puma/puma/compare/v8.0.1...v8.0.2</x:v>
       </x:c>
-      <x:c r="F241" s="4"/>
+      <x:c r="F241" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="242" ht="46" customHeight="1">
       <x:c r="A242" s="4" t="str">
@@ -5345,7 +6059,9 @@
       <x:c r="E242" s="4" t="str">
         <x:v>https://github.com/pymc-labs/pymc-marketing/compare/0.16.0...0.17.0</x:v>
       </x:c>
-      <x:c r="F242" s="4"/>
+      <x:c r="F242" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="243" ht="46" customHeight="1">
       <x:c r="A243" s="4" t="str">
@@ -5363,7 +6079,9 @@
       <x:c r="E243" s="4" t="str">
         <x:v>https://github.com/pymc-labs/pymc-marketing/compare/0.18.2...0.19.0</x:v>
       </x:c>
-      <x:c r="F243" s="4"/>
+      <x:c r="F243" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="244" ht="46" customHeight="1">
       <x:c r="A244" s="4" t="str">
@@ -5381,7 +6099,9 @@
       <x:c r="E244" s="4" t="str">
         <x:v>https://github.com/pymc-labs/pymc-marketing/compare/0.19.2...0.19.3</x:v>
       </x:c>
-      <x:c r="F244" s="4"/>
+      <x:c r="F244" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="245" ht="46" customHeight="1">
       <x:c r="A245" s="4" t="str">
@@ -5399,7 +6119,9 @@
       <x:c r="E245" s="4" t="str">
         <x:v>https://github.com/pymc-labs/pymc-marketing/compare/0.19.3...0.19.4</x:v>
       </x:c>
-      <x:c r="F245" s="4"/>
+      <x:c r="F245" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="246" ht="46" customHeight="1">
       <x:c r="A246" s="4" t="str">
@@ -5417,7 +6139,9 @@
       <x:c r="E246" s="4" t="str">
         <x:v>https://github.com/pymc-labs/pymc-marketing/compare/1.0.0...1.1.0</x:v>
       </x:c>
-      <x:c r="F246" s="4"/>
+      <x:c r="F246" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="247" ht="46" customHeight="1">
       <x:c r="A247" s="4" t="str">
@@ -5435,7 +6159,9 @@
       <x:c r="E247" s="4" t="str">
         <x:v>https://github.com/qiutongxue/oba-live-tool/compare/v1.5.11...v1.5.12</x:v>
       </x:c>
-      <x:c r="F247" s="4"/>
+      <x:c r="F247" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="248" ht="46" customHeight="1">
       <x:c r="A248" s="4" t="str">
@@ -5453,7 +6179,9 @@
       <x:c r="E248" s="4" t="str">
         <x:v>https://github.com/qiutongxue/oba-live-tool/compare/v1.5.12...v1.5.13</x:v>
       </x:c>
-      <x:c r="F248" s="4"/>
+      <x:c r="F248" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="249" ht="46" customHeight="1">
       <x:c r="A249" s="4" t="str">
@@ -5471,7 +6199,9 @@
       <x:c r="E249" s="4" t="str">
         <x:v>https://github.com/qiutongxue/oba-live-tool/compare/v1.5.16...v1.5.17</x:v>
       </x:c>
-      <x:c r="F249" s="4"/>
+      <x:c r="F249" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="250" ht="46" customHeight="1">
       <x:c r="A250" s="4" t="str">
@@ -5489,7 +6219,9 @@
       <x:c r="E250" s="4" t="str">
         <x:v>https://github.com/qiutongxue/oba-live-tool/compare/v1.5.22...v1.5.23</x:v>
       </x:c>
-      <x:c r="F250" s="4"/>
+      <x:c r="F250" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="251" ht="46" customHeight="1">
       <x:c r="A251" s="4" t="str">
@@ -5507,7 +6239,9 @@
       <x:c r="E251" s="4" t="str">
         <x:v>https://github.com/qiutongxue/oba-live-tool/compare/v1.6.1...v1.6.2</x:v>
       </x:c>
-      <x:c r="F251" s="4"/>
+      <x:c r="F251" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="252" ht="46" customHeight="1">
       <x:c r="A252" s="4" t="str">
@@ -5525,7 +6259,9 @@
       <x:c r="E252" s="4" t="str">
         <x:v>https://github.com/qiz029/dscode/compare/v0.4.0...v0.5.0</x:v>
       </x:c>
-      <x:c r="F252" s="4"/>
+      <x:c r="F252" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="253" ht="46" customHeight="1">
       <x:c r="A253" s="4" t="str">
@@ -5543,7 +6279,9 @@
       <x:c r="E253" s="4" t="str">
         <x:v>https://github.com/qiz029/dscode/compare/v0.7.8...v0.7.9</x:v>
       </x:c>
-      <x:c r="F253" s="4"/>
+      <x:c r="F253" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="254" ht="46" customHeight="1">
       <x:c r="A254" s="4" t="str">
@@ -5561,7 +6299,9 @@
       <x:c r="E254" s="4" t="str">
         <x:v>https://github.com/qiz029/dscode/compare/v0.7.12...v0.7.13</x:v>
       </x:c>
-      <x:c r="F254" s="4"/>
+      <x:c r="F254" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="255" ht="46" customHeight="1">
       <x:c r="A255" s="4" t="str">
@@ -5579,7 +6319,9 @@
       <x:c r="E255" s="4" t="str">
         <x:v>https://github.com/qiz029/dscode/compare/v0.7.24...v0.7.25</x:v>
       </x:c>
-      <x:c r="F255" s="4"/>
+      <x:c r="F255" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="256" ht="46" customHeight="1">
       <x:c r="A256" s="4" t="str">
@@ -5597,7 +6339,9 @@
       <x:c r="E256" s="4" t="str">
         <x:v>https://github.com/qiz029/dscode/compare/v0.7.30...v0.7.31</x:v>
       </x:c>
-      <x:c r="F256" s="4"/>
+      <x:c r="F256" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="257" ht="46" customHeight="1">
       <x:c r="A257" s="4" t="str">
@@ -5615,7 +6359,9 @@
       <x:c r="E257" s="4" t="str">
         <x:v>https://github.com/remorses/playwriter/compare/playwriter%400.0.41...playwriter%400.0.42</x:v>
       </x:c>
-      <x:c r="F257" s="4"/>
+      <x:c r="F257" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="258" ht="46" customHeight="1">
       <x:c r="A258" s="4" t="str">
@@ -5633,7 +6379,9 @@
       <x:c r="E258" s="4" t="str">
         <x:v>https://github.com/remorses/playwriter/compare/playwriter%400.0.45...playwriter%400.0.46</x:v>
       </x:c>
-      <x:c r="F258" s="4"/>
+      <x:c r="F258" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="259" ht="46" customHeight="1">
       <x:c r="A259" s="4" t="str">
@@ -5651,7 +6399,9 @@
       <x:c r="E259" s="4" t="str">
         <x:v>https://github.com/remorses/playwriter/compare/playwriter%400.0.50...playwriter%400.0.52</x:v>
       </x:c>
-      <x:c r="F259" s="4"/>
+      <x:c r="F259" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="260" ht="46" customHeight="1">
       <x:c r="A260" s="4" t="str">
@@ -5669,7 +6419,9 @@
       <x:c r="E260" s="4" t="str">
         <x:v>https://github.com/remorses/playwriter/compare/playwriter%400.0.62...playwriter%400.0.63</x:v>
       </x:c>
-      <x:c r="F260" s="4"/>
+      <x:c r="F260" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="261" ht="46" customHeight="1">
       <x:c r="A261" s="4" t="str">
@@ -5687,7 +6439,9 @@
       <x:c r="E261" s="4" t="str">
         <x:v>https://github.com/remorses/playwriter/compare/playwriter%400.0.63...playwriter%400.0.80</x:v>
       </x:c>
-      <x:c r="F261" s="4"/>
+      <x:c r="F261" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="262" ht="46" customHeight="1">
       <x:c r="A262" s="4" t="str">
@@ -5705,7 +6459,9 @@
       <x:c r="E262" s="4" t="str">
         <x:v>https://github.com/rhysd/actionlint/compare/v1.7.7...v1.7.8</x:v>
       </x:c>
-      <x:c r="F262" s="4"/>
+      <x:c r="F262" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="263" ht="46" customHeight="1">
       <x:c r="A263" s="4" t="str">
@@ -5723,7 +6479,9 @@
       <x:c r="E263" s="4" t="str">
         <x:v>https://github.com/rhysd/actionlint/compare/v1.7.8...v1.7.9</x:v>
       </x:c>
-      <x:c r="F263" s="4"/>
+      <x:c r="F263" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="264" ht="46" customHeight="1">
       <x:c r="A264" s="4" t="str">
@@ -5741,7 +6499,9 @@
       <x:c r="E264" s="4" t="str">
         <x:v>https://github.com/rhysd/actionlint/compare/v1.7.9...v1.7.10</x:v>
       </x:c>
-      <x:c r="F264" s="4"/>
+      <x:c r="F264" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="265" ht="46" customHeight="1">
       <x:c r="A265" s="4" t="str">
@@ -5759,7 +6519,9 @@
       <x:c r="E265" s="4" t="str">
         <x:v>https://github.com/rhysd/actionlint/compare/v1.7.10...v1.7.11</x:v>
       </x:c>
-      <x:c r="F265" s="4"/>
+      <x:c r="F265" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="266" ht="46" customHeight="1">
       <x:c r="A266" s="4" t="str">
@@ -5777,7 +6539,9 @@
       <x:c r="E266" s="4" t="str">
         <x:v>https://github.com/rhysd/actionlint/compare/v1.7.11...v1.7.12</x:v>
       </x:c>
-      <x:c r="F266" s="4"/>
+      <x:c r="F266" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="267" ht="46" customHeight="1">
       <x:c r="A267" s="4" t="str">
@@ -5795,7 +6559,9 @@
       <x:c r="E267" s="4" t="str">
         <x:v>https://github.com/superdoc/docx-editor/compare/v1.14.0...v1.15.0</x:v>
       </x:c>
-      <x:c r="F267" s="4"/>
+      <x:c r="F267" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="268" ht="46" customHeight="1">
       <x:c r="A268" s="4" t="str">
@@ -5813,7 +6579,9 @@
       <x:c r="E268" s="4" t="str">
         <x:v>https://github.com/superdoc/docx-editor/compare/template-builder-v1.3.0...cli-v0.5.1</x:v>
       </x:c>
-      <x:c r="F268" s="4"/>
+      <x:c r="F268" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="269" ht="46" customHeight="1">
       <x:c r="A269" s="4" t="str">
@@ -5831,7 +6599,9 @@
       <x:c r="E269" s="4" t="str">
         <x:v>https://github.com/superdoc/docx-editor/compare/sdk-v1.3.0...v1.24.2</x:v>
       </x:c>
-      <x:c r="F269" s="4"/>
+      <x:c r="F269" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="270" ht="46" customHeight="1">
       <x:c r="A270" s="4" t="str">
@@ -5849,7 +6619,9 @@
       <x:c r="E270" s="4" t="str">
         <x:v>https://github.com/superdoc/docx-editor/compare/sdk-v1.20.0...mcp-v0.16.0</x:v>
       </x:c>
-      <x:c r="F270" s="4"/>
+      <x:c r="F270" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="271" ht="46" customHeight="1">
       <x:c r="A271" s="4" t="str">
@@ -5867,7 +6639,9 @@
       <x:c r="E271" s="4" t="str">
         <x:v>https://github.com/superdoc/docx-editor/compare/react-v1.16.0...vscode-v2.17.0</x:v>
       </x:c>
-      <x:c r="F271" s="4"/>
+      <x:c r="F271" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="272" ht="46" customHeight="1">
       <x:c r="A272" s="4" t="str">
@@ -5885,7 +6659,9 @@
       <x:c r="E272" s="4" t="str">
         <x:v>https://github.com/unicode-org/icu4x/compare/ffi-artifacts/2025-08-13...icu%402.1.0</x:v>
       </x:c>
-      <x:c r="F272" s="4"/>
+      <x:c r="F272" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="273" ht="46" customHeight="1">
       <x:c r="A273" s="4" t="str">
@@ -5903,7 +6679,9 @@
       <x:c r="E273" s="4" t="str">
         <x:v>https://github.com/unicode-org/icu4x/compare/icu%402.1.0...ffi-artifacts/2025-12-12</x:v>
       </x:c>
-      <x:c r="F273" s="4"/>
+      <x:c r="F273" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="274" ht="46" customHeight="1">
       <x:c r="A274" s="4" t="str">
@@ -5921,7 +6699,9 @@
       <x:c r="E274" s="4" t="str">
         <x:v>https://github.com/unicode-org/icu4x/compare/ffi-artifacts/2025-12-12...icu%402.2.0</x:v>
       </x:c>
-      <x:c r="F274" s="4"/>
+      <x:c r="F274" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="275" ht="46" customHeight="1">
       <x:c r="A275" s="4" t="str">
@@ -5939,7 +6719,9 @@
       <x:c r="E275" s="4" t="str">
         <x:v>https://github.com/unicode-org/icu4x/compare/icu%402.2.0...icu%402.3.0</x:v>
       </x:c>
-      <x:c r="F275" s="4"/>
+      <x:c r="F275" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="276" ht="46" customHeight="1">
       <x:c r="A276" s="4" t="str">
@@ -5957,7 +6739,9 @@
       <x:c r="E276" s="4" t="str">
         <x:v>https://github.com/unicode-org/icu4x/compare/icu%402.3.0...icu%402.3.1</x:v>
       </x:c>
-      <x:c r="F276" s="4"/>
+      <x:c r="F276" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="277" ht="46" customHeight="1">
       <x:c r="A277" s="4" t="str">
@@ -5975,7 +6759,9 @@
       <x:c r="E277" s="4" t="str">
         <x:v>https://github.com/utkuozdemir/pv-migrate/compare/v2.2.1...v3.0.0</x:v>
       </x:c>
-      <x:c r="F277" s="4"/>
+      <x:c r="F277" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="278" ht="46" customHeight="1">
       <x:c r="A278" s="4" t="str">
@@ -5993,7 +6779,9 @@
       <x:c r="E278" s="4" t="str">
         <x:v>https://github.com/utkuozdemir/pv-migrate/compare/v3.0.0...v3.1.0</x:v>
       </x:c>
-      <x:c r="F278" s="4"/>
+      <x:c r="F278" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="279" ht="46" customHeight="1">
       <x:c r="A279" s="4" t="str">
@@ -6011,7 +6799,9 @@
       <x:c r="E279" s="4" t="str">
         <x:v>https://github.com/utkuozdemir/pv-migrate/compare/v3.4.0...v3.5.0</x:v>
       </x:c>
-      <x:c r="F279" s="4"/>
+      <x:c r="F279" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="280" ht="46" customHeight="1">
       <x:c r="A280" s="4" t="str">
@@ -6029,7 +6819,9 @@
       <x:c r="E280" s="4" t="str">
         <x:v>https://github.com/utkuozdemir/pv-migrate/compare/v3.6.0...v3.6.1</x:v>
       </x:c>
-      <x:c r="F280" s="4"/>
+      <x:c r="F280" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="281" ht="46" customHeight="1">
       <x:c r="A281" s="4" t="str">
@@ -6047,7 +6839,9 @@
       <x:c r="E281" s="4" t="str">
         <x:v>https://github.com/utkuozdemir/pv-migrate/compare/v3.6.1...v3.6.2</x:v>
       </x:c>
-      <x:c r="F281" s="4"/>
+      <x:c r="F281" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="282" ht="46" customHeight="1">
       <x:c r="A282" s="4" t="str">
@@ -6065,7 +6859,9 @@
       <x:c r="E282" s="4" t="str">
         <x:v>https://github.com/vergecurrency/verge/compare/v8.0.0...v8.0.1</x:v>
       </x:c>
-      <x:c r="F282" s="4"/>
+      <x:c r="F282" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="283" ht="46" customHeight="1">
       <x:c r="A283" s="4" t="str">
@@ -6083,7 +6879,9 @@
       <x:c r="E283" s="4" t="str">
         <x:v>https://github.com/vergecurrency/verge/compare/v8.0.1...v8.0.2</x:v>
       </x:c>
-      <x:c r="F283" s="4"/>
+      <x:c r="F283" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="284" ht="46" customHeight="1">
       <x:c r="A284" s="4" t="str">
@@ -6101,7 +6899,9 @@
       <x:c r="E284" s="4" t="str">
         <x:v>https://github.com/vergecurrency/verge/compare/v8.0.2...v8.0.3</x:v>
       </x:c>
-      <x:c r="F284" s="4"/>
+      <x:c r="F284" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="285" ht="46" customHeight="1">
       <x:c r="A285" s="4" t="str">
@@ -6119,7 +6919,9 @@
       <x:c r="E285" s="4" t="str">
         <x:v>https://github.com/vergecurrency/verge/compare/v26.5.0.0...v26.5.1</x:v>
       </x:c>
-      <x:c r="F285" s="4"/>
+      <x:c r="F285" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="286" ht="46" customHeight="1">
       <x:c r="A286" s="4" t="str">
@@ -6137,7 +6939,9 @@
       <x:c r="E286" s="4" t="str">
         <x:v>https://github.com/vergecurrency/verge/compare/v26.5.1...v26.7</x:v>
       </x:c>
-      <x:c r="F286" s="4"/>
+      <x:c r="F286" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="287" ht="46" customHeight="1">
       <x:c r="A287" s="4" t="str">
@@ -6155,7 +6959,9 @@
       <x:c r="E287" s="4" t="str">
         <x:v>https://github.com/vllm-project/llm-compressor/compare/0.7.1...0.8.0</x:v>
       </x:c>
-      <x:c r="F287" s="4"/>
+      <x:c r="F287" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="288" ht="46" customHeight="1">
       <x:c r="A288" s="4" t="str">
@@ -6173,7 +6979,9 @@
       <x:c r="E288" s="4" t="str">
         <x:v>https://github.com/vllm-project/llm-compressor/compare/0.8.0...0.8.1</x:v>
       </x:c>
-      <x:c r="F288" s="4"/>
+      <x:c r="F288" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="289" ht="46" customHeight="1">
       <x:c r="A289" s="4" t="str">
@@ -6191,7 +6999,9 @@
       <x:c r="E289" s="4" t="str">
         <x:v>https://github.com/vllm-project/llm-compressor/compare/0.10.0.1...0.10.0.2</x:v>
       </x:c>
-      <x:c r="F289" s="4"/>
+      <x:c r="F289" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="290" ht="46" customHeight="1">
       <x:c r="A290" s="4" t="str">
@@ -6209,7 +7019,9 @@
       <x:c r="E290" s="4" t="str">
         <x:v>https://github.com/vllm-project/llm-compressor/compare/0.7.1.4...0.9.0.4</x:v>
       </x:c>
-      <x:c r="F290" s="4"/>
+      <x:c r="F290" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="291" ht="46" customHeight="1">
       <x:c r="A291" s="4" t="str">
@@ -6227,7 +7039,9 @@
       <x:c r="E291" s="4" t="str">
         <x:v>https://github.com/vllm-project/llm-compressor/compare/0.10.0.3...0.12.0.1</x:v>
       </x:c>
-      <x:c r="F291" s="4"/>
+      <x:c r="F291" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="292" ht="46" customHeight="1">
       <x:c r="A292" s="4" t="str">
@@ -6245,7 +7059,9 @@
       <x:c r="E292" s="4" t="str">
         <x:v>https://github.com/yhan-sun/p2wlan/compare/v0.1.57...v0.1.58</x:v>
       </x:c>
-      <x:c r="F292" s="4"/>
+      <x:c r="F292" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="293" ht="46" customHeight="1">
       <x:c r="A293" s="4" t="str">
@@ -6263,7 +7079,9 @@
       <x:c r="E293" s="4" t="str">
         <x:v>https://github.com/yhan-sun/p2wlan/compare/v0.1.108...v0.1.109</x:v>
       </x:c>
-      <x:c r="F293" s="4"/>
+      <x:c r="F293" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="294" ht="46" customHeight="1">
       <x:c r="A294" s="4" t="str">
@@ -6281,7 +7099,9 @@
       <x:c r="E294" s="4" t="str">
         <x:v>https://github.com/yhan-sun/p2wlan/compare/v0.1.119...v0.1.120</x:v>
       </x:c>
-      <x:c r="F294" s="4"/>
+      <x:c r="F294" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="295" ht="46" customHeight="1">
       <x:c r="A295" s="4" t="str">
@@ -6299,7 +7119,9 @@
       <x:c r="E295" s="4" t="str">
         <x:v>https://github.com/yhan-sun/p2wlan/compare/v0.1.122...v0.1.123</x:v>
       </x:c>
-      <x:c r="F295" s="4"/>
+      <x:c r="F295" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="296" ht="46" customHeight="1">
       <x:c r="A296" s="4" t="str">
@@ -6317,7 +7139,9 @@
       <x:c r="E296" s="4" t="str">
         <x:v>https://github.com/yhan-sun/p2wlan/compare/v0.1.156...v0.1.157</x:v>
       </x:c>
-      <x:c r="F296" s="4"/>
+      <x:c r="F296" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="297" ht="46" customHeight="1">
       <x:c r="A297" s="4" t="str">
@@ -6335,7 +7159,9 @@
       <x:c r="E297" s="4" t="str">
         <x:v>https://github.com/zerx-lab/FluxDown/compare/cli-v0.1.57...mobile-v0.1.57</x:v>
       </x:c>
-      <x:c r="F297" s="4"/>
+      <x:c r="F297" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="298" ht="46" customHeight="1">
       <x:c r="A298" s="4" t="str">
@@ -6353,7 +7179,9 @@
       <x:c r="E298" s="4" t="str">
         <x:v>https://github.com/zerx-lab/FluxDown/compare/v0.1.59...extension-v0.2.0</x:v>
       </x:c>
-      <x:c r="F298" s="4"/>
+      <x:c r="F298" s="4" t="str">
+        <x:v>não</x:v>
+      </x:c>
     </x:row>
     <x:row r="299" ht="46" customHeight="1">
       <x:c r="A299" s="4" t="str">
@@ -6371,7 +7199,9 @@
       <x:c r="E299" s="4" t="str">
         <x:v>https://github.com/zerx-lab/FluxDown/compare/v0.2.0...cli-v0.2.1</x:v>
       </x:c>
-      <x:c r="F299" s="4"/>
+      <x:c r="F299" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="300" ht="46" customHeight="1">
       <x:c r="A300" s="4" t="str">
@@ -6389,7 +7219,9 @@
       <x:c r="E300" s="4" t="str">
         <x:v>https://github.com/zerx-lab/FluxDown/compare/cli-v0.3.0...mobile-v0.3.0</x:v>
       </x:c>
-      <x:c r="F300" s="4"/>
+      <x:c r="F300" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
     <x:row r="301" ht="46" customHeight="1">
       <x:c r="A301" s="4" t="str">
@@ -6407,7 +7239,9 @@
       <x:c r="E301" s="4" t="str">
         <x:v>https://github.com/zerx-lab/FluxDown/compare/server-v0.3.1...mobile-v0.3.1</x:v>
       </x:c>
-      <x:c r="F301" s="4"/>
+      <x:c r="F301" s="4" t="str">
+        <x:v>sim</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">

</xml_diff>